<commit_message>
[ROS-LL-v4.2.0] Add approved fields and correct reference links
</commit_message>
<xml_diff>
--- a/form_reporting_templates/ROS-LL/v4.2.0/Form-ROS-LL-v4.2.0.xlsx
+++ b/form_reporting_templates/ROS-LL/v4.2.0/Form-ROS-LL-v4.2.0.xlsx
@@ -18234,7 +18234,7 @@
   <hyperlinks>
     <hyperlink ref="I2" r:id="rId1" location="weightMeasurements" xr:uid="{779410D5-0433-4C34-84B6-98A10CA2B249}"/>
     <hyperlink ref="K2" r:id="rId2" location="weightMeasurementTools" xr:uid="{EB80831C-DDCE-4E4D-A605-160D23E19E90}"/>
-    <hyperlink ref="E2" r:id="rId3" location="typesOfFate" xr:uid="{F8152E0B-B9D5-4E81-A374-4985E0AF2D58}"/>
+    <hyperlink ref="E2" r:id="rId3" xr:uid="{F8152E0B-B9D5-4E81-A374-4985E0AF2D58}" location="fateTypes"/>
     <hyperlink ref="F2" r:id="rId4" location="fates" xr:uid="{5DE917A8-1BC5-48A5-BE95-3206B5EEB7AC}"/>
     <hyperlink ref="D1" r:id="rIdSpecies420_6" xr:uid="{7915C09B-5FFF-4B7E-84FB-D8B7D31EA643}" location="allSpecies"/>
     <hyperlink ref="G1:G2" r:id="rId6" location="samplingMethodsForCatchEstimation" display="SAMPLING_METHOD" xr:uid="{C3154411-BFD2-3A41-99A0-2ECAAC5C9F3C}"/>
@@ -23412,7 +23412,7 @@
     <hyperlink ref="E1:E2" r:id="rId1" location="samplingPeriods" display="SAMPLING_PERIOD" xr:uid="{C0407D03-A3E9-4479-BB66-8329070009A1}"/>
     <hyperlink ref="V2" r:id="rId2" location="depredationSources" xr:uid="{5248D097-7FB7-4BF7-908D-893A3BF91D4F}"/>
     <hyperlink ref="W2" r:id="rIdSpecies420_8" xr:uid="{16A7B676-4806-46E0-B05E-266794DC9A6F}" location="predatorSpecies"/>
-    <hyperlink ref="F1:F2" r:id="rId4" location="samplingMethodsForSamplingCollection" display="SAMPLING_METHOD" xr:uid="{863AF79D-449A-4B35-AC8D-9C415D8A32B9}"/>
+    <hyperlink ref="F1:F2" r:id="rId4" display="SAMPLING_METHOD" xr:uid="{863AF79D-449A-4B35-AC8D-9C415D8A32B9}" location="samplingMethodsForSamplingCollections"/>
     <hyperlink ref="I2" r:id="rId5" location="lengthMeasurementTools" xr:uid="{776CD30A-4D78-4230-9891-093ADBA1D96D}"/>
     <hyperlink ref="L2" r:id="rId6" location="lengthMeasurementTools" xr:uid="{3DE19339-45B9-47B8-B5FB-D4012AD9C532}"/>
     <hyperlink ref="G2" r:id="rIdV420_G2" xr:uid="{4F273766-A7DB-428C-A222-09DB4E6495A6}" location="allMeasurements"/>
@@ -27973,7 +27973,7 @@
   </dataValidations>
   <hyperlinks>
     <hyperlink ref="G1:G2" r:id="rId1" location="gearInteractions" display="GEAR_INTERACTION" xr:uid="{4D21FAB4-D1ED-49FA-A8E9-1A452DA8E255}"/>
-    <hyperlink ref="H1:H2" r:id="rId2" location="hookTypes" display="HOOK_TYPE" xr:uid="{FC3E5B48-31F4-4395-B266-CAE8F0285CBE}"/>
+    <hyperlink ref="H1:H2" r:id="rId2" display="HOOK_TYPE" xr:uid="{FC3E5B48-31F4-4395-B266-CAE8F0285CBE}" location="hookAndTerminalDevices"/>
     <hyperlink ref="I2" r:id="rIdV420_I2" xr:uid="{A5E5073A-7EA6-4050-99BD-3A2C3C210913}" location="baitConditions"/>
     <hyperlink ref="M1:M2" r:id="rId4" location="dehookerTypes" display="DEHOOKER_DEVICE" xr:uid="{223FF70D-0F50-400C-91DF-40947EEFC402}"/>
     <hyperlink ref="K2" r:id="rId5" location="lineMaterialTypes" xr:uid="{8BD5CD8E-6908-4DE0-9B07-7CCA6FB5C649}"/>
@@ -39834,12 +39834,12 @@
   <hyperlinks>
     <hyperlink ref="C2:C3" r:id="rId1" location="countries" display="FLAG_OR_CHARTERING_STATE" xr:uid="{DA9CE3B1-74F9-4268-98AF-290FAC660EAD}"/>
     <hyperlink ref="G2" r:id="rId2" location="countries" display="COUNTRY_CODE" xr:uid="{4939BF01-E483-4611-A010-33B090D54E39}"/>
-    <hyperlink ref="J1" r:id="rId3" location="targetSpecies" display="SPECIES_1_CODE" xr:uid="{E9AF38ED-FD60-4672-8F14-35015A129362}"/>
+    <hyperlink ref="J1" r:id="rId3" display="SPECIES_1_CODE" xr:uid="{E9AF38ED-FD60-4672-8F14-35015A129362}" location="targetSpecies"/>
     <hyperlink ref="M3" r:id="rId4" location="countries" xr:uid="{10913ED0-4328-48D4-A042-6201D824CECA}"/>
     <hyperlink ref="O3" r:id="rId5" location="countries" xr:uid="{3CF4C3FC-91EE-45A1-9C82-1871A741D19A}"/>
     <hyperlink ref="H2" r:id="rIdV420_H2" display="PORT_CODE" xr:uid="{C4D05E8A-B26C-4196-BF44-6883318591EB}" location="ports"/>
     <hyperlink ref="K2:K3" r:id="rId7" location="gears" display="MAIN_FISHING_GEAR" xr:uid="{ADDD99C7-B692-4517-AF11-C5F4715C3781}"/>
-    <hyperlink ref="H2:H3" r:id="rId8" location="Ports" display="PORT" xr:uid="{4BCE8909-E3DB-4961-B5C5-527D383D1926}"/>
+    <hyperlink ref="H2:H3" r:id="rId8" display="PORT" xr:uid="{4BCE8909-E3DB-4961-B5C5-527D383D1926}" location="ports"/>
     <hyperlink ref="J1:J3" r:id="rId9" location="targetSpecies" display="LICENSED_TARGET_SPECIES" xr:uid="{8145BEA5-06D1-4F1F-890E-1ACE66463F94}"/>
     <hyperlink ref="G2:G3" r:id="rId10" location="countries" display="COUNTRY" xr:uid="{40B25D40-1383-402F-BBDE-DC1B90768417}"/>
   </hyperlinks>
@@ -51485,7 +51485,7 @@
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="D2:D3" r:id="rId1" location="hullMaterialTypes" display="HULL_MATERIAL" xr:uid="{67410786-49B8-4FAC-82C7-693110607986}"/>
+    <hyperlink ref="D2:D3" r:id="rId1" display="HULL_MATERIAL" xr:uid="{67410786-49B8-4FAC-82C7-693110607986}" location="hullMaterialTypes"/>
     <hyperlink ref="L3" r:id="rId2" location="fishPreservationMethods" xr:uid="{1302D005-C0D4-48F4-9067-8DB21E13C99E}"/>
     <hyperlink ref="M3" r:id="rId3" location="fishPreservationMethods" xr:uid="{EEBE083B-4312-4FA4-A951-C9F9A824B321}"/>
     <hyperlink ref="N3" r:id="rId4" location="fishPreservationMethods" xr:uid="{30064C75-6784-480A-88EC-D543ED3C0DC7}"/>
@@ -59209,7 +59209,7 @@
   <sheetPr>
     <tabColor theme="8" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:AB203"/>
+  <dimension ref="A1:AG203"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="20.6640625" style="3" customWidth="1"/>
@@ -59229,17 +59229,22 @@
     <col min="15" max="15" width="9.1640625" style="3"/>
     <col min="16" max="16" width="27.83203125" style="3" customWidth="1"/>
     <col min="17" max="17" width="27.5" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="33.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="9.1640625" style="3"/>
-    <col min="20" max="20" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="11.5" style="3" customWidth="1"/>
-    <col min="22" max="22" width="12.6640625" style="3" customWidth="1"/>
-    <col min="23" max="23" width="30" style="3" customWidth="1"/>
-    <col min="24" max="24" width="30" style="3" customWidth="1"/>
-    <col min="25" max="25" width="15.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="15.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="15.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="15.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="32" style="3" customWidth="1"/>
+    <col min="19" max="19" width="32" style="3" customWidth="1"/>
+    <col min="20" max="20" width="32" style="3" customWidth="1"/>
+    <col min="21" max="21" width="32" style="3" customWidth="1"/>
+    <col min="22" max="22" width="33.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="32" style="3" customWidth="1"/>
+    <col min="24" max="24" width="9.1640625" style="3"/>
+    <col min="25" max="25" width="14.6640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="11.5" style="3" customWidth="1"/>
+    <col min="27" max="27" width="12.6640625" style="3" customWidth="1"/>
+    <col min="28" max="28" width="30" style="3" customWidth="1"/>
+    <col min="29" max="29" width="30" style="3" customWidth="1"/>
+    <col min="30" max="30" width="15.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="15.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="15.83203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="15.83203125" style="3" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" s="41" customFormat="1" x14ac:dyDescent="0.2">
@@ -59280,33 +59285,58 @@
       <c r="Q1" s="103" t="s">
         <v>236</v>
       </c>
-      <c r="R1" s="85" t="s">
+      <c r="R1" s="103" t="inlineStr">
+        <is>
+          <t>NUMBER_RADIO_DHAN_BUOYS_SET</t>
+        </is>
+      </c>
+      <c r="S1" s="85" t="inlineStr">
+        <is>
+          <t>FLOATLINE_LENGTH_1_M</t>
+        </is>
+      </c>
+      <c r="T1" s="103" t="inlineStr">
+        <is>
+          <t>FLOATLINE_LENGTH_2_M</t>
+        </is>
+      </c>
+      <c r="U1" s="103" t="inlineStr">
+        <is>
+          <t>FLOATLINE_LENGTH_3_M</t>
+        </is>
+      </c>
+      <c r="V1" s="85" t="s">
         <v>237</v>
       </c>
-      <c r="S1" s="85" t="s">
+      <c r="W1" s="103" t="inlineStr">
+        <is>
+          <t>DISTANCE_BETWEEN_BRANCHLINES_M</t>
+        </is>
+      </c>
+      <c r="X1" s="85" t="s">
         <v>243</v>
       </c>
-      <c r="T1" s="85"/>
-      <c r="U1" s="122" t="s">
+      <c r="Y1" s="85"/>
+      <c r="Z1" s="122" t="s">
         <v>244</v>
       </c>
-      <c r="V1" s="123"/>
-      <c r="W1" s="122" t="inlineStr">
+      <c r="AA1" s="123"/>
+      <c r="AB1" s="122" t="inlineStr">
         <is>
           <t>BRANCHLINE_LENGTH_MIN_M</t>
         </is>
       </c>
-      <c r="X1" s="122" t="inlineStr">
+      <c r="AC1" s="122" t="inlineStr">
         <is>
           <t>BRANCHLINE_LENGTH_MAX_M</t>
         </is>
       </c>
-      <c r="Y1" s="85" t="s">
+      <c r="AD1" s="85" t="s">
         <v>242</v>
       </c>
-      <c r="Z1" s="85"/>
-      <c r="AA1" s="85"/>
-      <c r="AB1" s="85"/>
+      <c r="AE1" s="85"/>
+      <c r="AF1" s="85"/>
+      <c r="AG1" s="85"/>
     </row>
     <row r="2" s="41" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A2" s="73"/>
@@ -59334,17 +59364,22 @@
       <c r="O2" s="84"/>
       <c r="P2" s="85"/>
       <c r="Q2" s="103"/>
-      <c r="R2" s="85"/>
+      <c r="R2" s="103"/>
       <c r="S2" s="85"/>
-      <c r="T2" s="85"/>
-      <c r="U2" s="80"/>
-      <c r="V2" s="82"/>
-      <c r="W2" s="80"/>
-      <c r="X2" s="80"/>
+      <c r="T2" s="103"/>
+      <c r="U2" s="103"/>
+      <c r="V2" s="85"/>
+      <c r="W2" s="103"/>
+      <c r="X2" s="85"/>
       <c r="Y2" s="85"/>
-      <c r="Z2" s="85"/>
-      <c r="AA2" s="85"/>
-      <c r="AB2" s="85"/>
+      <c r="Z2" s="80"/>
+      <c r="AA2" s="82"/>
+      <c r="AB2" s="80"/>
+      <c r="AC2" s="80"/>
+      <c r="AD2" s="85"/>
+      <c r="AE2" s="85"/>
+      <c r="AF2" s="85"/>
+      <c r="AG2" s="85"/>
     </row>
     <row r="3" s="41" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A3" s="74"/>
@@ -59382,31 +59417,36 @@
       </c>
       <c r="P3" s="85"/>
       <c r="Q3" s="103"/>
-      <c r="R3" s="85"/>
-      <c r="S3" s="30" t="s">
+      <c r="V3" s="85"/>
+      <c r="X3" s="30" t="s">
         <v>50</v>
       </c>
-      <c r="T3" s="33" t="s">
+      <c r="R3" s="103"/>
+      <c r="S3" s="85"/>
+      <c r="T3" s="103"/>
+      <c r="U3" s="103"/>
+      <c r="W3" s="103"/>
+      <c r="Y3" s="33" t="s">
         <v>15</v>
       </c>
-      <c r="U3" s="57" t="s">
+      <c r="Z3" s="57" t="s">
         <v>23</v>
       </c>
-      <c r="V3" s="30" t="s">
+      <c r="AA3" s="30" t="s">
         <v>51</v>
       </c>
-      <c r="W3" s="30"/>
-      <c r="X3" s="30"/>
-      <c r="Y3" s="42" t="s">
+      <c r="AB3" s="30"/>
+      <c r="AC3" s="30"/>
+      <c r="AD3" s="42" t="s">
         <v>238</v>
       </c>
-      <c r="Z3" s="36" t="s">
+      <c r="AE3" s="36" t="s">
         <v>239</v>
       </c>
-      <c r="AA3" s="36" t="s">
+      <c r="AF3" s="36" t="s">
         <v>240</v>
       </c>
-      <c r="AB3" s="36" t="s">
+      <c r="AG3" s="36" t="s">
         <v>241</v>
       </c>
     </row>
@@ -59439,6 +59479,11 @@
       <c r="Z4" s="2"/>
       <c r="AA4" s="2"/>
       <c r="AB4" s="2"/>
+      <c r="AC4" s="2"/>
+      <c r="AD4" s="2"/>
+      <c r="AE4" s="2"/>
+      <c r="AF4" s="2"/>
+      <c r="AG4" s="2"/>
     </row>
     <row r="5" x14ac:dyDescent="0.2">
       <c r="A5" s="2"/>
@@ -59469,6 +59514,11 @@
       <c r="Z5" s="2"/>
       <c r="AA5" s="2"/>
       <c r="AB5" s="2"/>
+      <c r="AC5" s="2"/>
+      <c r="AD5" s="2"/>
+      <c r="AE5" s="2"/>
+      <c r="AF5" s="2"/>
+      <c r="AG5" s="2"/>
     </row>
     <row r="6" x14ac:dyDescent="0.2">
       <c r="A6" s="2"/>
@@ -59499,6 +59549,11 @@
       <c r="Z6" s="2"/>
       <c r="AA6" s="2"/>
       <c r="AB6" s="2"/>
+      <c r="AC6" s="2"/>
+      <c r="AD6" s="2"/>
+      <c r="AE6" s="2"/>
+      <c r="AF6" s="2"/>
+      <c r="AG6" s="2"/>
     </row>
     <row r="7" x14ac:dyDescent="0.2">
       <c r="A7" s="2"/>
@@ -59529,6 +59584,11 @@
       <c r="Z7" s="2"/>
       <c r="AA7" s="2"/>
       <c r="AB7" s="2"/>
+      <c r="AC7" s="2"/>
+      <c r="AD7" s="2"/>
+      <c r="AE7" s="2"/>
+      <c r="AF7" s="2"/>
+      <c r="AG7" s="2"/>
     </row>
     <row r="8" x14ac:dyDescent="0.2">
       <c r="A8" s="2"/>
@@ -59559,6 +59619,11 @@
       <c r="Z8" s="2"/>
       <c r="AA8" s="2"/>
       <c r="AB8" s="2"/>
+      <c r="AC8" s="2"/>
+      <c r="AD8" s="2"/>
+      <c r="AE8" s="2"/>
+      <c r="AF8" s="2"/>
+      <c r="AG8" s="2"/>
     </row>
     <row r="9" x14ac:dyDescent="0.2">
       <c r="A9" s="2"/>
@@ -59589,6 +59654,11 @@
       <c r="Z9" s="2"/>
       <c r="AA9" s="2"/>
       <c r="AB9" s="2"/>
+      <c r="AC9" s="2"/>
+      <c r="AD9" s="2"/>
+      <c r="AE9" s="2"/>
+      <c r="AF9" s="2"/>
+      <c r="AG9" s="2"/>
     </row>
     <row r="10" x14ac:dyDescent="0.2">
       <c r="A10" s="2"/>
@@ -59619,6 +59689,11 @@
       <c r="Z10" s="2"/>
       <c r="AA10" s="2"/>
       <c r="AB10" s="2"/>
+      <c r="AC10" s="2"/>
+      <c r="AD10" s="2"/>
+      <c r="AE10" s="2"/>
+      <c r="AF10" s="2"/>
+      <c r="AG10" s="2"/>
     </row>
     <row r="11" x14ac:dyDescent="0.2">
       <c r="A11" s="2"/>
@@ -59649,6 +59724,11 @@
       <c r="Z11" s="2"/>
       <c r="AA11" s="2"/>
       <c r="AB11" s="2"/>
+      <c r="AC11" s="2"/>
+      <c r="AD11" s="2"/>
+      <c r="AE11" s="2"/>
+      <c r="AF11" s="2"/>
+      <c r="AG11" s="2"/>
     </row>
     <row r="12" x14ac:dyDescent="0.2">
       <c r="A12" s="2"/>
@@ -59679,6 +59759,11 @@
       <c r="Z12" s="2"/>
       <c r="AA12" s="2"/>
       <c r="AB12" s="2"/>
+      <c r="AC12" s="2"/>
+      <c r="AD12" s="2"/>
+      <c r="AE12" s="2"/>
+      <c r="AF12" s="2"/>
+      <c r="AG12" s="2"/>
     </row>
     <row r="13" x14ac:dyDescent="0.2">
       <c r="A13" s="2"/>
@@ -59709,6 +59794,11 @@
       <c r="Z13" s="2"/>
       <c r="AA13" s="2"/>
       <c r="AB13" s="2"/>
+      <c r="AC13" s="2"/>
+      <c r="AD13" s="2"/>
+      <c r="AE13" s="2"/>
+      <c r="AF13" s="2"/>
+      <c r="AG13" s="2"/>
     </row>
     <row r="14" x14ac:dyDescent="0.2">
       <c r="A14" s="2"/>
@@ -59739,6 +59829,11 @@
       <c r="Z14" s="2"/>
       <c r="AA14" s="2"/>
       <c r="AB14" s="2"/>
+      <c r="AC14" s="2"/>
+      <c r="AD14" s="2"/>
+      <c r="AE14" s="2"/>
+      <c r="AF14" s="2"/>
+      <c r="AG14" s="2"/>
     </row>
     <row r="15" x14ac:dyDescent="0.2">
       <c r="A15" s="2"/>
@@ -59769,6 +59864,11 @@
       <c r="Z15" s="2"/>
       <c r="AA15" s="2"/>
       <c r="AB15" s="2"/>
+      <c r="AC15" s="2"/>
+      <c r="AD15" s="2"/>
+      <c r="AE15" s="2"/>
+      <c r="AF15" s="2"/>
+      <c r="AG15" s="2"/>
     </row>
     <row r="16" x14ac:dyDescent="0.2">
       <c r="A16" s="2"/>
@@ -59799,6 +59899,11 @@
       <c r="Z16" s="2"/>
       <c r="AA16" s="2"/>
       <c r="AB16" s="2"/>
+      <c r="AC16" s="2"/>
+      <c r="AD16" s="2"/>
+      <c r="AE16" s="2"/>
+      <c r="AF16" s="2"/>
+      <c r="AG16" s="2"/>
     </row>
     <row r="17" x14ac:dyDescent="0.2">
       <c r="A17" s="2"/>
@@ -59829,6 +59934,11 @@
       <c r="Z17" s="2"/>
       <c r="AA17" s="2"/>
       <c r="AB17" s="2"/>
+      <c r="AC17" s="2"/>
+      <c r="AD17" s="2"/>
+      <c r="AE17" s="2"/>
+      <c r="AF17" s="2"/>
+      <c r="AG17" s="2"/>
     </row>
     <row r="18" x14ac:dyDescent="0.2">
       <c r="A18" s="2"/>
@@ -59859,6 +59969,11 @@
       <c r="Z18" s="2"/>
       <c r="AA18" s="2"/>
       <c r="AB18" s="2"/>
+      <c r="AC18" s="2"/>
+      <c r="AD18" s="2"/>
+      <c r="AE18" s="2"/>
+      <c r="AF18" s="2"/>
+      <c r="AG18" s="2"/>
     </row>
     <row r="19" x14ac:dyDescent="0.2">
       <c r="A19" s="2"/>
@@ -59889,6 +60004,11 @@
       <c r="Z19" s="2"/>
       <c r="AA19" s="2"/>
       <c r="AB19" s="2"/>
+      <c r="AC19" s="2"/>
+      <c r="AD19" s="2"/>
+      <c r="AE19" s="2"/>
+      <c r="AF19" s="2"/>
+      <c r="AG19" s="2"/>
     </row>
     <row r="20" x14ac:dyDescent="0.2">
       <c r="A20" s="2"/>
@@ -59919,6 +60039,11 @@
       <c r="Z20" s="2"/>
       <c r="AA20" s="2"/>
       <c r="AB20" s="2"/>
+      <c r="AC20" s="2"/>
+      <c r="AD20" s="2"/>
+      <c r="AE20" s="2"/>
+      <c r="AF20" s="2"/>
+      <c r="AG20" s="2"/>
     </row>
     <row r="21" x14ac:dyDescent="0.2">
       <c r="A21" s="2"/>
@@ -59949,6 +60074,11 @@
       <c r="Z21" s="2"/>
       <c r="AA21" s="2"/>
       <c r="AB21" s="2"/>
+      <c r="AC21" s="2"/>
+      <c r="AD21" s="2"/>
+      <c r="AE21" s="2"/>
+      <c r="AF21" s="2"/>
+      <c r="AG21" s="2"/>
     </row>
     <row r="22" x14ac:dyDescent="0.2">
       <c r="A22" s="2"/>
@@ -59979,6 +60109,11 @@
       <c r="Z22" s="2"/>
       <c r="AA22" s="2"/>
       <c r="AB22" s="2"/>
+      <c r="AC22" s="2"/>
+      <c r="AD22" s="2"/>
+      <c r="AE22" s="2"/>
+      <c r="AF22" s="2"/>
+      <c r="AG22" s="2"/>
     </row>
     <row r="23" x14ac:dyDescent="0.2">
       <c r="A23" s="2"/>
@@ -60009,6 +60144,11 @@
       <c r="Z23" s="2"/>
       <c r="AA23" s="2"/>
       <c r="AB23" s="2"/>
+      <c r="AC23" s="2"/>
+      <c r="AD23" s="2"/>
+      <c r="AE23" s="2"/>
+      <c r="AF23" s="2"/>
+      <c r="AG23" s="2"/>
     </row>
     <row r="24" x14ac:dyDescent="0.2">
       <c r="A24" s="2"/>
@@ -60039,6 +60179,11 @@
       <c r="Z24" s="2"/>
       <c r="AA24" s="2"/>
       <c r="AB24" s="2"/>
+      <c r="AC24" s="2"/>
+      <c r="AD24" s="2"/>
+      <c r="AE24" s="2"/>
+      <c r="AF24" s="2"/>
+      <c r="AG24" s="2"/>
     </row>
     <row r="25" x14ac:dyDescent="0.2">
       <c r="A25" s="2"/>
@@ -60069,6 +60214,11 @@
       <c r="Z25" s="2"/>
       <c r="AA25" s="2"/>
       <c r="AB25" s="2"/>
+      <c r="AC25" s="2"/>
+      <c r="AD25" s="2"/>
+      <c r="AE25" s="2"/>
+      <c r="AF25" s="2"/>
+      <c r="AG25" s="2"/>
     </row>
     <row r="26" x14ac:dyDescent="0.2">
       <c r="A26" s="2"/>
@@ -60099,6 +60249,11 @@
       <c r="Z26" s="2"/>
       <c r="AA26" s="2"/>
       <c r="AB26" s="2"/>
+      <c r="AC26" s="2"/>
+      <c r="AD26" s="2"/>
+      <c r="AE26" s="2"/>
+      <c r="AF26" s="2"/>
+      <c r="AG26" s="2"/>
     </row>
     <row r="27" x14ac:dyDescent="0.2">
       <c r="A27" s="2"/>
@@ -60129,6 +60284,11 @@
       <c r="Z27" s="2"/>
       <c r="AA27" s="2"/>
       <c r="AB27" s="2"/>
+      <c r="AC27" s="2"/>
+      <c r="AD27" s="2"/>
+      <c r="AE27" s="2"/>
+      <c r="AF27" s="2"/>
+      <c r="AG27" s="2"/>
     </row>
     <row r="28" x14ac:dyDescent="0.2">
       <c r="A28" s="2"/>
@@ -60159,6 +60319,11 @@
       <c r="Z28" s="2"/>
       <c r="AA28" s="2"/>
       <c r="AB28" s="2"/>
+      <c r="AC28" s="2"/>
+      <c r="AD28" s="2"/>
+      <c r="AE28" s="2"/>
+      <c r="AF28" s="2"/>
+      <c r="AG28" s="2"/>
     </row>
     <row r="29" x14ac:dyDescent="0.2">
       <c r="A29" s="2"/>
@@ -60189,6 +60354,11 @@
       <c r="Z29" s="2"/>
       <c r="AA29" s="2"/>
       <c r="AB29" s="2"/>
+      <c r="AC29" s="2"/>
+      <c r="AD29" s="2"/>
+      <c r="AE29" s="2"/>
+      <c r="AF29" s="2"/>
+      <c r="AG29" s="2"/>
     </row>
     <row r="30" x14ac:dyDescent="0.2">
       <c r="A30" s="2"/>
@@ -60219,6 +60389,11 @@
       <c r="Z30" s="2"/>
       <c r="AA30" s="2"/>
       <c r="AB30" s="2"/>
+      <c r="AC30" s="2"/>
+      <c r="AD30" s="2"/>
+      <c r="AE30" s="2"/>
+      <c r="AF30" s="2"/>
+      <c r="AG30" s="2"/>
     </row>
     <row r="31" x14ac:dyDescent="0.2">
       <c r="A31" s="2"/>
@@ -60249,6 +60424,11 @@
       <c r="Z31" s="2"/>
       <c r="AA31" s="2"/>
       <c r="AB31" s="2"/>
+      <c r="AC31" s="2"/>
+      <c r="AD31" s="2"/>
+      <c r="AE31" s="2"/>
+      <c r="AF31" s="2"/>
+      <c r="AG31" s="2"/>
     </row>
     <row r="32" x14ac:dyDescent="0.2">
       <c r="A32" s="2"/>
@@ -60279,6 +60459,11 @@
       <c r="Z32" s="2"/>
       <c r="AA32" s="2"/>
       <c r="AB32" s="2"/>
+      <c r="AC32" s="2"/>
+      <c r="AD32" s="2"/>
+      <c r="AE32" s="2"/>
+      <c r="AF32" s="2"/>
+      <c r="AG32" s="2"/>
     </row>
     <row r="33" x14ac:dyDescent="0.2">
       <c r="A33" s="2"/>
@@ -60309,6 +60494,11 @@
       <c r="Z33" s="2"/>
       <c r="AA33" s="2"/>
       <c r="AB33" s="2"/>
+      <c r="AC33" s="2"/>
+      <c r="AD33" s="2"/>
+      <c r="AE33" s="2"/>
+      <c r="AF33" s="2"/>
+      <c r="AG33" s="2"/>
     </row>
     <row r="34" x14ac:dyDescent="0.2">
       <c r="A34" s="2"/>
@@ -60339,6 +60529,11 @@
       <c r="Z34" s="2"/>
       <c r="AA34" s="2"/>
       <c r="AB34" s="2"/>
+      <c r="AC34" s="2"/>
+      <c r="AD34" s="2"/>
+      <c r="AE34" s="2"/>
+      <c r="AF34" s="2"/>
+      <c r="AG34" s="2"/>
     </row>
     <row r="35" x14ac:dyDescent="0.2">
       <c r="A35" s="2"/>
@@ -60369,6 +60564,11 @@
       <c r="Z35" s="2"/>
       <c r="AA35" s="2"/>
       <c r="AB35" s="2"/>
+      <c r="AC35" s="2"/>
+      <c r="AD35" s="2"/>
+      <c r="AE35" s="2"/>
+      <c r="AF35" s="2"/>
+      <c r="AG35" s="2"/>
     </row>
     <row r="36" x14ac:dyDescent="0.2">
       <c r="A36" s="2"/>
@@ -60399,6 +60599,11 @@
       <c r="Z36" s="2"/>
       <c r="AA36" s="2"/>
       <c r="AB36" s="2"/>
+      <c r="AC36" s="2"/>
+      <c r="AD36" s="2"/>
+      <c r="AE36" s="2"/>
+      <c r="AF36" s="2"/>
+      <c r="AG36" s="2"/>
     </row>
     <row r="37" x14ac:dyDescent="0.2">
       <c r="A37" s="2"/>
@@ -60429,6 +60634,11 @@
       <c r="Z37" s="2"/>
       <c r="AA37" s="2"/>
       <c r="AB37" s="2"/>
+      <c r="AC37" s="2"/>
+      <c r="AD37" s="2"/>
+      <c r="AE37" s="2"/>
+      <c r="AF37" s="2"/>
+      <c r="AG37" s="2"/>
     </row>
     <row r="38" x14ac:dyDescent="0.2">
       <c r="A38" s="2"/>
@@ -60459,6 +60669,11 @@
       <c r="Z38" s="2"/>
       <c r="AA38" s="2"/>
       <c r="AB38" s="2"/>
+      <c r="AC38" s="2"/>
+      <c r="AD38" s="2"/>
+      <c r="AE38" s="2"/>
+      <c r="AF38" s="2"/>
+      <c r="AG38" s="2"/>
     </row>
     <row r="39" x14ac:dyDescent="0.2">
       <c r="A39" s="2"/>
@@ -60489,6 +60704,11 @@
       <c r="Z39" s="2"/>
       <c r="AA39" s="2"/>
       <c r="AB39" s="2"/>
+      <c r="AC39" s="2"/>
+      <c r="AD39" s="2"/>
+      <c r="AE39" s="2"/>
+      <c r="AF39" s="2"/>
+      <c r="AG39" s="2"/>
     </row>
     <row r="40" x14ac:dyDescent="0.2">
       <c r="A40" s="2"/>
@@ -60519,6 +60739,11 @@
       <c r="Z40" s="2"/>
       <c r="AA40" s="2"/>
       <c r="AB40" s="2"/>
+      <c r="AC40" s="2"/>
+      <c r="AD40" s="2"/>
+      <c r="AE40" s="2"/>
+      <c r="AF40" s="2"/>
+      <c r="AG40" s="2"/>
     </row>
     <row r="41" x14ac:dyDescent="0.2">
       <c r="A41" s="2"/>
@@ -60549,6 +60774,11 @@
       <c r="Z41" s="2"/>
       <c r="AA41" s="2"/>
       <c r="AB41" s="2"/>
+      <c r="AC41" s="2"/>
+      <c r="AD41" s="2"/>
+      <c r="AE41" s="2"/>
+      <c r="AF41" s="2"/>
+      <c r="AG41" s="2"/>
     </row>
     <row r="42" x14ac:dyDescent="0.2">
       <c r="A42" s="2"/>
@@ -60579,6 +60809,11 @@
       <c r="Z42" s="2"/>
       <c r="AA42" s="2"/>
       <c r="AB42" s="2"/>
+      <c r="AC42" s="2"/>
+      <c r="AD42" s="2"/>
+      <c r="AE42" s="2"/>
+      <c r="AF42" s="2"/>
+      <c r="AG42" s="2"/>
     </row>
     <row r="43" x14ac:dyDescent="0.2">
       <c r="A43" s="2"/>
@@ -60609,6 +60844,11 @@
       <c r="Z43" s="2"/>
       <c r="AA43" s="2"/>
       <c r="AB43" s="2"/>
+      <c r="AC43" s="2"/>
+      <c r="AD43" s="2"/>
+      <c r="AE43" s="2"/>
+      <c r="AF43" s="2"/>
+      <c r="AG43" s="2"/>
     </row>
     <row r="44" x14ac:dyDescent="0.2">
       <c r="A44" s="2"/>
@@ -60639,6 +60879,11 @@
       <c r="Z44" s="2"/>
       <c r="AA44" s="2"/>
       <c r="AB44" s="2"/>
+      <c r="AC44" s="2"/>
+      <c r="AD44" s="2"/>
+      <c r="AE44" s="2"/>
+      <c r="AF44" s="2"/>
+      <c r="AG44" s="2"/>
     </row>
     <row r="45" x14ac:dyDescent="0.2">
       <c r="A45" s="2"/>
@@ -60669,6 +60914,11 @@
       <c r="Z45" s="2"/>
       <c r="AA45" s="2"/>
       <c r="AB45" s="2"/>
+      <c r="AC45" s="2"/>
+      <c r="AD45" s="2"/>
+      <c r="AE45" s="2"/>
+      <c r="AF45" s="2"/>
+      <c r="AG45" s="2"/>
     </row>
     <row r="46" x14ac:dyDescent="0.2">
       <c r="A46" s="2"/>
@@ -60699,6 +60949,11 @@
       <c r="Z46" s="2"/>
       <c r="AA46" s="2"/>
       <c r="AB46" s="2"/>
+      <c r="AC46" s="2"/>
+      <c r="AD46" s="2"/>
+      <c r="AE46" s="2"/>
+      <c r="AF46" s="2"/>
+      <c r="AG46" s="2"/>
     </row>
     <row r="47" x14ac:dyDescent="0.2">
       <c r="A47" s="2"/>
@@ -60729,6 +60984,11 @@
       <c r="Z47" s="2"/>
       <c r="AA47" s="2"/>
       <c r="AB47" s="2"/>
+      <c r="AC47" s="2"/>
+      <c r="AD47" s="2"/>
+      <c r="AE47" s="2"/>
+      <c r="AF47" s="2"/>
+      <c r="AG47" s="2"/>
     </row>
     <row r="48" x14ac:dyDescent="0.2">
       <c r="A48" s="2"/>
@@ -60759,6 +61019,11 @@
       <c r="Z48" s="2"/>
       <c r="AA48" s="2"/>
       <c r="AB48" s="2"/>
+      <c r="AC48" s="2"/>
+      <c r="AD48" s="2"/>
+      <c r="AE48" s="2"/>
+      <c r="AF48" s="2"/>
+      <c r="AG48" s="2"/>
     </row>
     <row r="49" x14ac:dyDescent="0.2">
       <c r="A49" s="2"/>
@@ -60789,6 +61054,11 @@
       <c r="Z49" s="2"/>
       <c r="AA49" s="2"/>
       <c r="AB49" s="2"/>
+      <c r="AC49" s="2"/>
+      <c r="AD49" s="2"/>
+      <c r="AE49" s="2"/>
+      <c r="AF49" s="2"/>
+      <c r="AG49" s="2"/>
     </row>
     <row r="50" x14ac:dyDescent="0.2">
       <c r="A50" s="2"/>
@@ -60819,6 +61089,11 @@
       <c r="Z50" s="2"/>
       <c r="AA50" s="2"/>
       <c r="AB50" s="2"/>
+      <c r="AC50" s="2"/>
+      <c r="AD50" s="2"/>
+      <c r="AE50" s="2"/>
+      <c r="AF50" s="2"/>
+      <c r="AG50" s="2"/>
     </row>
     <row r="51" x14ac:dyDescent="0.2">
       <c r="A51" s="2"/>
@@ -60849,6 +61124,11 @@
       <c r="Z51" s="2"/>
       <c r="AA51" s="2"/>
       <c r="AB51" s="2"/>
+      <c r="AC51" s="2"/>
+      <c r="AD51" s="2"/>
+      <c r="AE51" s="2"/>
+      <c r="AF51" s="2"/>
+      <c r="AG51" s="2"/>
     </row>
     <row r="52" x14ac:dyDescent="0.2">
       <c r="A52" s="2"/>
@@ -60879,6 +61159,11 @@
       <c r="Z52" s="2"/>
       <c r="AA52" s="2"/>
       <c r="AB52" s="2"/>
+      <c r="AC52" s="2"/>
+      <c r="AD52" s="2"/>
+      <c r="AE52" s="2"/>
+      <c r="AF52" s="2"/>
+      <c r="AG52" s="2"/>
     </row>
     <row r="53" x14ac:dyDescent="0.2">
       <c r="A53" s="2"/>
@@ -60909,6 +61194,11 @@
       <c r="Z53" s="2"/>
       <c r="AA53" s="2"/>
       <c r="AB53" s="2"/>
+      <c r="AC53" s="2"/>
+      <c r="AD53" s="2"/>
+      <c r="AE53" s="2"/>
+      <c r="AF53" s="2"/>
+      <c r="AG53" s="2"/>
     </row>
     <row r="54" x14ac:dyDescent="0.2">
       <c r="A54" s="2"/>
@@ -60939,6 +61229,11 @@
       <c r="Z54" s="2"/>
       <c r="AA54" s="2"/>
       <c r="AB54" s="2"/>
+      <c r="AC54" s="2"/>
+      <c r="AD54" s="2"/>
+      <c r="AE54" s="2"/>
+      <c r="AF54" s="2"/>
+      <c r="AG54" s="2"/>
     </row>
     <row r="55" x14ac:dyDescent="0.2">
       <c r="A55" s="2"/>
@@ -60969,6 +61264,11 @@
       <c r="Z55" s="2"/>
       <c r="AA55" s="2"/>
       <c r="AB55" s="2"/>
+      <c r="AC55" s="2"/>
+      <c r="AD55" s="2"/>
+      <c r="AE55" s="2"/>
+      <c r="AF55" s="2"/>
+      <c r="AG55" s="2"/>
     </row>
     <row r="56" x14ac:dyDescent="0.2">
       <c r="A56" s="2"/>
@@ -60999,6 +61299,11 @@
       <c r="Z56" s="2"/>
       <c r="AA56" s="2"/>
       <c r="AB56" s="2"/>
+      <c r="AC56" s="2"/>
+      <c r="AD56" s="2"/>
+      <c r="AE56" s="2"/>
+      <c r="AF56" s="2"/>
+      <c r="AG56" s="2"/>
     </row>
     <row r="57" x14ac:dyDescent="0.2">
       <c r="A57" s="2"/>
@@ -61029,6 +61334,11 @@
       <c r="Z57" s="2"/>
       <c r="AA57" s="2"/>
       <c r="AB57" s="2"/>
+      <c r="AC57" s="2"/>
+      <c r="AD57" s="2"/>
+      <c r="AE57" s="2"/>
+      <c r="AF57" s="2"/>
+      <c r="AG57" s="2"/>
     </row>
     <row r="58" x14ac:dyDescent="0.2">
       <c r="A58" s="2"/>
@@ -61059,6 +61369,11 @@
       <c r="Z58" s="2"/>
       <c r="AA58" s="2"/>
       <c r="AB58" s="2"/>
+      <c r="AC58" s="2"/>
+      <c r="AD58" s="2"/>
+      <c r="AE58" s="2"/>
+      <c r="AF58" s="2"/>
+      <c r="AG58" s="2"/>
     </row>
     <row r="59" x14ac:dyDescent="0.2">
       <c r="A59" s="2"/>
@@ -61089,6 +61404,11 @@
       <c r="Z59" s="2"/>
       <c r="AA59" s="2"/>
       <c r="AB59" s="2"/>
+      <c r="AC59" s="2"/>
+      <c r="AD59" s="2"/>
+      <c r="AE59" s="2"/>
+      <c r="AF59" s="2"/>
+      <c r="AG59" s="2"/>
     </row>
     <row r="60" x14ac:dyDescent="0.2">
       <c r="A60" s="2"/>
@@ -61119,6 +61439,11 @@
       <c r="Z60" s="2"/>
       <c r="AA60" s="2"/>
       <c r="AB60" s="2"/>
+      <c r="AC60" s="2"/>
+      <c r="AD60" s="2"/>
+      <c r="AE60" s="2"/>
+      <c r="AF60" s="2"/>
+      <c r="AG60" s="2"/>
     </row>
     <row r="61" x14ac:dyDescent="0.2">
       <c r="A61" s="2"/>
@@ -61149,6 +61474,11 @@
       <c r="Z61" s="2"/>
       <c r="AA61" s="2"/>
       <c r="AB61" s="2"/>
+      <c r="AC61" s="2"/>
+      <c r="AD61" s="2"/>
+      <c r="AE61" s="2"/>
+      <c r="AF61" s="2"/>
+      <c r="AG61" s="2"/>
     </row>
     <row r="62" x14ac:dyDescent="0.2">
       <c r="A62" s="2"/>
@@ -61179,6 +61509,11 @@
       <c r="Z62" s="2"/>
       <c r="AA62" s="2"/>
       <c r="AB62" s="2"/>
+      <c r="AC62" s="2"/>
+      <c r="AD62" s="2"/>
+      <c r="AE62" s="2"/>
+      <c r="AF62" s="2"/>
+      <c r="AG62" s="2"/>
     </row>
     <row r="63" x14ac:dyDescent="0.2">
       <c r="A63" s="2"/>
@@ -61209,6 +61544,11 @@
       <c r="Z63" s="2"/>
       <c r="AA63" s="2"/>
       <c r="AB63" s="2"/>
+      <c r="AC63" s="2"/>
+      <c r="AD63" s="2"/>
+      <c r="AE63" s="2"/>
+      <c r="AF63" s="2"/>
+      <c r="AG63" s="2"/>
     </row>
     <row r="64" x14ac:dyDescent="0.2">
       <c r="A64" s="2"/>
@@ -61239,6 +61579,11 @@
       <c r="Z64" s="2"/>
       <c r="AA64" s="2"/>
       <c r="AB64" s="2"/>
+      <c r="AC64" s="2"/>
+      <c r="AD64" s="2"/>
+      <c r="AE64" s="2"/>
+      <c r="AF64" s="2"/>
+      <c r="AG64" s="2"/>
     </row>
     <row r="65" x14ac:dyDescent="0.2">
       <c r="A65" s="2"/>
@@ -61269,6 +61614,11 @@
       <c r="Z65" s="2"/>
       <c r="AA65" s="2"/>
       <c r="AB65" s="2"/>
+      <c r="AC65" s="2"/>
+      <c r="AD65" s="2"/>
+      <c r="AE65" s="2"/>
+      <c r="AF65" s="2"/>
+      <c r="AG65" s="2"/>
     </row>
     <row r="66" x14ac:dyDescent="0.2">
       <c r="A66" s="2"/>
@@ -61299,6 +61649,11 @@
       <c r="Z66" s="2"/>
       <c r="AA66" s="2"/>
       <c r="AB66" s="2"/>
+      <c r="AC66" s="2"/>
+      <c r="AD66" s="2"/>
+      <c r="AE66" s="2"/>
+      <c r="AF66" s="2"/>
+      <c r="AG66" s="2"/>
     </row>
     <row r="67" x14ac:dyDescent="0.2">
       <c r="A67" s="2"/>
@@ -61329,6 +61684,11 @@
       <c r="Z67" s="2"/>
       <c r="AA67" s="2"/>
       <c r="AB67" s="2"/>
+      <c r="AC67" s="2"/>
+      <c r="AD67" s="2"/>
+      <c r="AE67" s="2"/>
+      <c r="AF67" s="2"/>
+      <c r="AG67" s="2"/>
     </row>
     <row r="68" x14ac:dyDescent="0.2">
       <c r="A68" s="2"/>
@@ -61359,6 +61719,11 @@
       <c r="Z68" s="2"/>
       <c r="AA68" s="2"/>
       <c r="AB68" s="2"/>
+      <c r="AC68" s="2"/>
+      <c r="AD68" s="2"/>
+      <c r="AE68" s="2"/>
+      <c r="AF68" s="2"/>
+      <c r="AG68" s="2"/>
     </row>
     <row r="69" x14ac:dyDescent="0.2">
       <c r="A69" s="2"/>
@@ -61389,6 +61754,11 @@
       <c r="Z69" s="2"/>
       <c r="AA69" s="2"/>
       <c r="AB69" s="2"/>
+      <c r="AC69" s="2"/>
+      <c r="AD69" s="2"/>
+      <c r="AE69" s="2"/>
+      <c r="AF69" s="2"/>
+      <c r="AG69" s="2"/>
     </row>
     <row r="70" x14ac:dyDescent="0.2">
       <c r="A70" s="2"/>
@@ -61419,6 +61789,11 @@
       <c r="Z70" s="2"/>
       <c r="AA70" s="2"/>
       <c r="AB70" s="2"/>
+      <c r="AC70" s="2"/>
+      <c r="AD70" s="2"/>
+      <c r="AE70" s="2"/>
+      <c r="AF70" s="2"/>
+      <c r="AG70" s="2"/>
     </row>
     <row r="71" x14ac:dyDescent="0.2">
       <c r="A71" s="2"/>
@@ -61449,6 +61824,11 @@
       <c r="Z71" s="2"/>
       <c r="AA71" s="2"/>
       <c r="AB71" s="2"/>
+      <c r="AC71" s="2"/>
+      <c r="AD71" s="2"/>
+      <c r="AE71" s="2"/>
+      <c r="AF71" s="2"/>
+      <c r="AG71" s="2"/>
     </row>
     <row r="72" x14ac:dyDescent="0.2">
       <c r="A72" s="2"/>
@@ -61479,6 +61859,11 @@
       <c r="Z72" s="2"/>
       <c r="AA72" s="2"/>
       <c r="AB72" s="2"/>
+      <c r="AC72" s="2"/>
+      <c r="AD72" s="2"/>
+      <c r="AE72" s="2"/>
+      <c r="AF72" s="2"/>
+      <c r="AG72" s="2"/>
     </row>
     <row r="73" x14ac:dyDescent="0.2">
       <c r="A73" s="2"/>
@@ -61509,6 +61894,11 @@
       <c r="Z73" s="2"/>
       <c r="AA73" s="2"/>
       <c r="AB73" s="2"/>
+      <c r="AC73" s="2"/>
+      <c r="AD73" s="2"/>
+      <c r="AE73" s="2"/>
+      <c r="AF73" s="2"/>
+      <c r="AG73" s="2"/>
     </row>
     <row r="74" x14ac:dyDescent="0.2">
       <c r="A74" s="2"/>
@@ -61539,6 +61929,11 @@
       <c r="Z74" s="2"/>
       <c r="AA74" s="2"/>
       <c r="AB74" s="2"/>
+      <c r="AC74" s="2"/>
+      <c r="AD74" s="2"/>
+      <c r="AE74" s="2"/>
+      <c r="AF74" s="2"/>
+      <c r="AG74" s="2"/>
     </row>
     <row r="75" x14ac:dyDescent="0.2">
       <c r="A75" s="2"/>
@@ -61569,6 +61964,11 @@
       <c r="Z75" s="2"/>
       <c r="AA75" s="2"/>
       <c r="AB75" s="2"/>
+      <c r="AC75" s="2"/>
+      <c r="AD75" s="2"/>
+      <c r="AE75" s="2"/>
+      <c r="AF75" s="2"/>
+      <c r="AG75" s="2"/>
     </row>
     <row r="76" x14ac:dyDescent="0.2">
       <c r="A76" s="2"/>
@@ -61599,6 +61999,11 @@
       <c r="Z76" s="2"/>
       <c r="AA76" s="2"/>
       <c r="AB76" s="2"/>
+      <c r="AC76" s="2"/>
+      <c r="AD76" s="2"/>
+      <c r="AE76" s="2"/>
+      <c r="AF76" s="2"/>
+      <c r="AG76" s="2"/>
     </row>
     <row r="77" x14ac:dyDescent="0.2">
       <c r="A77" s="2"/>
@@ -61629,6 +62034,11 @@
       <c r="Z77" s="2"/>
       <c r="AA77" s="2"/>
       <c r="AB77" s="2"/>
+      <c r="AC77" s="2"/>
+      <c r="AD77" s="2"/>
+      <c r="AE77" s="2"/>
+      <c r="AF77" s="2"/>
+      <c r="AG77" s="2"/>
     </row>
     <row r="78" x14ac:dyDescent="0.2">
       <c r="A78" s="2"/>
@@ -61659,6 +62069,11 @@
       <c r="Z78" s="2"/>
       <c r="AA78" s="2"/>
       <c r="AB78" s="2"/>
+      <c r="AC78" s="2"/>
+      <c r="AD78" s="2"/>
+      <c r="AE78" s="2"/>
+      <c r="AF78" s="2"/>
+      <c r="AG78" s="2"/>
     </row>
     <row r="79" x14ac:dyDescent="0.2">
       <c r="A79" s="2"/>
@@ -61689,6 +62104,11 @@
       <c r="Z79" s="2"/>
       <c r="AA79" s="2"/>
       <c r="AB79" s="2"/>
+      <c r="AC79" s="2"/>
+      <c r="AD79" s="2"/>
+      <c r="AE79" s="2"/>
+      <c r="AF79" s="2"/>
+      <c r="AG79" s="2"/>
     </row>
     <row r="80" x14ac:dyDescent="0.2">
       <c r="A80" s="2"/>
@@ -61719,6 +62139,11 @@
       <c r="Z80" s="2"/>
       <c r="AA80" s="2"/>
       <c r="AB80" s="2"/>
+      <c r="AC80" s="2"/>
+      <c r="AD80" s="2"/>
+      <c r="AE80" s="2"/>
+      <c r="AF80" s="2"/>
+      <c r="AG80" s="2"/>
     </row>
     <row r="81" x14ac:dyDescent="0.2">
       <c r="A81" s="2"/>
@@ -61749,6 +62174,11 @@
       <c r="Z81" s="2"/>
       <c r="AA81" s="2"/>
       <c r="AB81" s="2"/>
+      <c r="AC81" s="2"/>
+      <c r="AD81" s="2"/>
+      <c r="AE81" s="2"/>
+      <c r="AF81" s="2"/>
+      <c r="AG81" s="2"/>
     </row>
     <row r="82" x14ac:dyDescent="0.2">
       <c r="A82" s="2"/>
@@ -61779,6 +62209,11 @@
       <c r="Z82" s="2"/>
       <c r="AA82" s="2"/>
       <c r="AB82" s="2"/>
+      <c r="AC82" s="2"/>
+      <c r="AD82" s="2"/>
+      <c r="AE82" s="2"/>
+      <c r="AF82" s="2"/>
+      <c r="AG82" s="2"/>
     </row>
     <row r="83" x14ac:dyDescent="0.2">
       <c r="A83" s="2"/>
@@ -61809,6 +62244,11 @@
       <c r="Z83" s="2"/>
       <c r="AA83" s="2"/>
       <c r="AB83" s="2"/>
+      <c r="AC83" s="2"/>
+      <c r="AD83" s="2"/>
+      <c r="AE83" s="2"/>
+      <c r="AF83" s="2"/>
+      <c r="AG83" s="2"/>
     </row>
     <row r="84" x14ac:dyDescent="0.2">
       <c r="A84" s="2"/>
@@ -61839,6 +62279,11 @@
       <c r="Z84" s="2"/>
       <c r="AA84" s="2"/>
       <c r="AB84" s="2"/>
+      <c r="AC84" s="2"/>
+      <c r="AD84" s="2"/>
+      <c r="AE84" s="2"/>
+      <c r="AF84" s="2"/>
+      <c r="AG84" s="2"/>
     </row>
     <row r="85" x14ac:dyDescent="0.2">
       <c r="A85" s="2"/>
@@ -61869,6 +62314,11 @@
       <c r="Z85" s="2"/>
       <c r="AA85" s="2"/>
       <c r="AB85" s="2"/>
+      <c r="AC85" s="2"/>
+      <c r="AD85" s="2"/>
+      <c r="AE85" s="2"/>
+      <c r="AF85" s="2"/>
+      <c r="AG85" s="2"/>
     </row>
     <row r="86" x14ac:dyDescent="0.2">
       <c r="A86" s="2"/>
@@ -61899,6 +62349,11 @@
       <c r="Z86" s="2"/>
       <c r="AA86" s="2"/>
       <c r="AB86" s="2"/>
+      <c r="AC86" s="2"/>
+      <c r="AD86" s="2"/>
+      <c r="AE86" s="2"/>
+      <c r="AF86" s="2"/>
+      <c r="AG86" s="2"/>
     </row>
     <row r="87" x14ac:dyDescent="0.2">
       <c r="A87" s="2"/>
@@ -61929,6 +62384,11 @@
       <c r="Z87" s="2"/>
       <c r="AA87" s="2"/>
       <c r="AB87" s="2"/>
+      <c r="AC87" s="2"/>
+      <c r="AD87" s="2"/>
+      <c r="AE87" s="2"/>
+      <c r="AF87" s="2"/>
+      <c r="AG87" s="2"/>
     </row>
     <row r="88" x14ac:dyDescent="0.2">
       <c r="A88" s="2"/>
@@ -61959,6 +62419,11 @@
       <c r="Z88" s="2"/>
       <c r="AA88" s="2"/>
       <c r="AB88" s="2"/>
+      <c r="AC88" s="2"/>
+      <c r="AD88" s="2"/>
+      <c r="AE88" s="2"/>
+      <c r="AF88" s="2"/>
+      <c r="AG88" s="2"/>
     </row>
     <row r="89" x14ac:dyDescent="0.2">
       <c r="A89" s="2"/>
@@ -61989,6 +62454,11 @@
       <c r="Z89" s="2"/>
       <c r="AA89" s="2"/>
       <c r="AB89" s="2"/>
+      <c r="AC89" s="2"/>
+      <c r="AD89" s="2"/>
+      <c r="AE89" s="2"/>
+      <c r="AF89" s="2"/>
+      <c r="AG89" s="2"/>
     </row>
     <row r="90" x14ac:dyDescent="0.2">
       <c r="A90" s="2"/>
@@ -62019,6 +62489,11 @@
       <c r="Z90" s="2"/>
       <c r="AA90" s="2"/>
       <c r="AB90" s="2"/>
+      <c r="AC90" s="2"/>
+      <c r="AD90" s="2"/>
+      <c r="AE90" s="2"/>
+      <c r="AF90" s="2"/>
+      <c r="AG90" s="2"/>
     </row>
     <row r="91" x14ac:dyDescent="0.2">
       <c r="A91" s="2"/>
@@ -62049,6 +62524,11 @@
       <c r="Z91" s="2"/>
       <c r="AA91" s="2"/>
       <c r="AB91" s="2"/>
+      <c r="AC91" s="2"/>
+      <c r="AD91" s="2"/>
+      <c r="AE91" s="2"/>
+      <c r="AF91" s="2"/>
+      <c r="AG91" s="2"/>
     </row>
     <row r="92" x14ac:dyDescent="0.2">
       <c r="A92" s="2"/>
@@ -62079,6 +62559,11 @@
       <c r="Z92" s="2"/>
       <c r="AA92" s="2"/>
       <c r="AB92" s="2"/>
+      <c r="AC92" s="2"/>
+      <c r="AD92" s="2"/>
+      <c r="AE92" s="2"/>
+      <c r="AF92" s="2"/>
+      <c r="AG92" s="2"/>
     </row>
     <row r="93" x14ac:dyDescent="0.2">
       <c r="A93" s="2"/>
@@ -62109,6 +62594,11 @@
       <c r="Z93" s="2"/>
       <c r="AA93" s="2"/>
       <c r="AB93" s="2"/>
+      <c r="AC93" s="2"/>
+      <c r="AD93" s="2"/>
+      <c r="AE93" s="2"/>
+      <c r="AF93" s="2"/>
+      <c r="AG93" s="2"/>
     </row>
     <row r="94" x14ac:dyDescent="0.2">
       <c r="A94" s="2"/>
@@ -62139,6 +62629,11 @@
       <c r="Z94" s="2"/>
       <c r="AA94" s="2"/>
       <c r="AB94" s="2"/>
+      <c r="AC94" s="2"/>
+      <c r="AD94" s="2"/>
+      <c r="AE94" s="2"/>
+      <c r="AF94" s="2"/>
+      <c r="AG94" s="2"/>
     </row>
     <row r="95" x14ac:dyDescent="0.2">
       <c r="A95" s="2"/>
@@ -62169,6 +62664,11 @@
       <c r="Z95" s="2"/>
       <c r="AA95" s="2"/>
       <c r="AB95" s="2"/>
+      <c r="AC95" s="2"/>
+      <c r="AD95" s="2"/>
+      <c r="AE95" s="2"/>
+      <c r="AF95" s="2"/>
+      <c r="AG95" s="2"/>
     </row>
     <row r="96" x14ac:dyDescent="0.2">
       <c r="A96" s="2"/>
@@ -62199,6 +62699,11 @@
       <c r="Z96" s="2"/>
       <c r="AA96" s="2"/>
       <c r="AB96" s="2"/>
+      <c r="AC96" s="2"/>
+      <c r="AD96" s="2"/>
+      <c r="AE96" s="2"/>
+      <c r="AF96" s="2"/>
+      <c r="AG96" s="2"/>
     </row>
     <row r="97" x14ac:dyDescent="0.2">
       <c r="A97" s="2"/>
@@ -62229,6 +62734,11 @@
       <c r="Z97" s="2"/>
       <c r="AA97" s="2"/>
       <c r="AB97" s="2"/>
+      <c r="AC97" s="2"/>
+      <c r="AD97" s="2"/>
+      <c r="AE97" s="2"/>
+      <c r="AF97" s="2"/>
+      <c r="AG97" s="2"/>
     </row>
     <row r="98" x14ac:dyDescent="0.2">
       <c r="A98" s="2"/>
@@ -62259,6 +62769,11 @@
       <c r="Z98" s="2"/>
       <c r="AA98" s="2"/>
       <c r="AB98" s="2"/>
+      <c r="AC98" s="2"/>
+      <c r="AD98" s="2"/>
+      <c r="AE98" s="2"/>
+      <c r="AF98" s="2"/>
+      <c r="AG98" s="2"/>
     </row>
     <row r="99" x14ac:dyDescent="0.2">
       <c r="A99" s="2"/>
@@ -62289,6 +62804,11 @@
       <c r="Z99" s="2"/>
       <c r="AA99" s="2"/>
       <c r="AB99" s="2"/>
+      <c r="AC99" s="2"/>
+      <c r="AD99" s="2"/>
+      <c r="AE99" s="2"/>
+      <c r="AF99" s="2"/>
+      <c r="AG99" s="2"/>
     </row>
     <row r="100" x14ac:dyDescent="0.2">
       <c r="A100" s="2"/>
@@ -62319,6 +62839,11 @@
       <c r="Z100" s="2"/>
       <c r="AA100" s="2"/>
       <c r="AB100" s="2"/>
+      <c r="AC100" s="2"/>
+      <c r="AD100" s="2"/>
+      <c r="AE100" s="2"/>
+      <c r="AF100" s="2"/>
+      <c r="AG100" s="2"/>
     </row>
     <row r="101" x14ac:dyDescent="0.2">
       <c r="A101" s="2"/>
@@ -62349,6 +62874,11 @@
       <c r="Z101" s="2"/>
       <c r="AA101" s="2"/>
       <c r="AB101" s="2"/>
+      <c r="AC101" s="2"/>
+      <c r="AD101" s="2"/>
+      <c r="AE101" s="2"/>
+      <c r="AF101" s="2"/>
+      <c r="AG101" s="2"/>
     </row>
     <row r="102" x14ac:dyDescent="0.2">
       <c r="A102" s="2"/>
@@ -62379,6 +62909,11 @@
       <c r="Z102" s="2"/>
       <c r="AA102" s="2"/>
       <c r="AB102" s="2"/>
+      <c r="AC102" s="2"/>
+      <c r="AD102" s="2"/>
+      <c r="AE102" s="2"/>
+      <c r="AF102" s="2"/>
+      <c r="AG102" s="2"/>
     </row>
     <row r="103" x14ac:dyDescent="0.2">
       <c r="A103" s="2"/>
@@ -62409,6 +62944,11 @@
       <c r="Z103" s="2"/>
       <c r="AA103" s="2"/>
       <c r="AB103" s="2"/>
+      <c r="AC103" s="2"/>
+      <c r="AD103" s="2"/>
+      <c r="AE103" s="2"/>
+      <c r="AF103" s="2"/>
+      <c r="AG103" s="2"/>
     </row>
     <row r="104" x14ac:dyDescent="0.2">
       <c r="A104" s="2"/>
@@ -62439,6 +62979,11 @@
       <c r="Z104" s="2"/>
       <c r="AA104" s="2"/>
       <c r="AB104" s="2"/>
+      <c r="AC104" s="2"/>
+      <c r="AD104" s="2"/>
+      <c r="AE104" s="2"/>
+      <c r="AF104" s="2"/>
+      <c r="AG104" s="2"/>
     </row>
     <row r="105" x14ac:dyDescent="0.2">
       <c r="A105" s="2"/>
@@ -62469,6 +63014,11 @@
       <c r="Z105" s="2"/>
       <c r="AA105" s="2"/>
       <c r="AB105" s="2"/>
+      <c r="AC105" s="2"/>
+      <c r="AD105" s="2"/>
+      <c r="AE105" s="2"/>
+      <c r="AF105" s="2"/>
+      <c r="AG105" s="2"/>
     </row>
     <row r="106" x14ac:dyDescent="0.2">
       <c r="A106" s="2"/>
@@ -62499,6 +63049,11 @@
       <c r="Z106" s="2"/>
       <c r="AA106" s="2"/>
       <c r="AB106" s="2"/>
+      <c r="AC106" s="2"/>
+      <c r="AD106" s="2"/>
+      <c r="AE106" s="2"/>
+      <c r="AF106" s="2"/>
+      <c r="AG106" s="2"/>
     </row>
     <row r="107" x14ac:dyDescent="0.2">
       <c r="A107" s="2"/>
@@ -62529,6 +63084,11 @@
       <c r="Z107" s="2"/>
       <c r="AA107" s="2"/>
       <c r="AB107" s="2"/>
+      <c r="AC107" s="2"/>
+      <c r="AD107" s="2"/>
+      <c r="AE107" s="2"/>
+      <c r="AF107" s="2"/>
+      <c r="AG107" s="2"/>
     </row>
     <row r="108" x14ac:dyDescent="0.2">
       <c r="A108" s="2"/>
@@ -62559,6 +63119,11 @@
       <c r="Z108" s="2"/>
       <c r="AA108" s="2"/>
       <c r="AB108" s="2"/>
+      <c r="AC108" s="2"/>
+      <c r="AD108" s="2"/>
+      <c r="AE108" s="2"/>
+      <c r="AF108" s="2"/>
+      <c r="AG108" s="2"/>
     </row>
     <row r="109" x14ac:dyDescent="0.2">
       <c r="A109" s="2"/>
@@ -62589,6 +63154,11 @@
       <c r="Z109" s="2"/>
       <c r="AA109" s="2"/>
       <c r="AB109" s="2"/>
+      <c r="AC109" s="2"/>
+      <c r="AD109" s="2"/>
+      <c r="AE109" s="2"/>
+      <c r="AF109" s="2"/>
+      <c r="AG109" s="2"/>
     </row>
     <row r="110" x14ac:dyDescent="0.2">
       <c r="A110" s="2"/>
@@ -62619,6 +63189,11 @@
       <c r="Z110" s="2"/>
       <c r="AA110" s="2"/>
       <c r="AB110" s="2"/>
+      <c r="AC110" s="2"/>
+      <c r="AD110" s="2"/>
+      <c r="AE110" s="2"/>
+      <c r="AF110" s="2"/>
+      <c r="AG110" s="2"/>
     </row>
     <row r="111" x14ac:dyDescent="0.2">
       <c r="A111" s="2"/>
@@ -62649,6 +63224,11 @@
       <c r="Z111" s="2"/>
       <c r="AA111" s="2"/>
       <c r="AB111" s="2"/>
+      <c r="AC111" s="2"/>
+      <c r="AD111" s="2"/>
+      <c r="AE111" s="2"/>
+      <c r="AF111" s="2"/>
+      <c r="AG111" s="2"/>
     </row>
     <row r="112" x14ac:dyDescent="0.2">
       <c r="A112" s="2"/>
@@ -62679,6 +63259,11 @@
       <c r="Z112" s="2"/>
       <c r="AA112" s="2"/>
       <c r="AB112" s="2"/>
+      <c r="AC112" s="2"/>
+      <c r="AD112" s="2"/>
+      <c r="AE112" s="2"/>
+      <c r="AF112" s="2"/>
+      <c r="AG112" s="2"/>
     </row>
     <row r="113" x14ac:dyDescent="0.2">
       <c r="A113" s="2"/>
@@ -62709,6 +63294,11 @@
       <c r="Z113" s="2"/>
       <c r="AA113" s="2"/>
       <c r="AB113" s="2"/>
+      <c r="AC113" s="2"/>
+      <c r="AD113" s="2"/>
+      <c r="AE113" s="2"/>
+      <c r="AF113" s="2"/>
+      <c r="AG113" s="2"/>
     </row>
     <row r="114" x14ac:dyDescent="0.2">
       <c r="A114" s="2"/>
@@ -62739,6 +63329,11 @@
       <c r="Z114" s="2"/>
       <c r="AA114" s="2"/>
       <c r="AB114" s="2"/>
+      <c r="AC114" s="2"/>
+      <c r="AD114" s="2"/>
+      <c r="AE114" s="2"/>
+      <c r="AF114" s="2"/>
+      <c r="AG114" s="2"/>
     </row>
     <row r="115" x14ac:dyDescent="0.2">
       <c r="A115" s="2"/>
@@ -62769,6 +63364,11 @@
       <c r="Z115" s="2"/>
       <c r="AA115" s="2"/>
       <c r="AB115" s="2"/>
+      <c r="AC115" s="2"/>
+      <c r="AD115" s="2"/>
+      <c r="AE115" s="2"/>
+      <c r="AF115" s="2"/>
+      <c r="AG115" s="2"/>
     </row>
     <row r="116" x14ac:dyDescent="0.2">
       <c r="A116" s="2"/>
@@ -62799,6 +63399,11 @@
       <c r="Z116" s="2"/>
       <c r="AA116" s="2"/>
       <c r="AB116" s="2"/>
+      <c r="AC116" s="2"/>
+      <c r="AD116" s="2"/>
+      <c r="AE116" s="2"/>
+      <c r="AF116" s="2"/>
+      <c r="AG116" s="2"/>
     </row>
     <row r="117" x14ac:dyDescent="0.2">
       <c r="A117" s="2"/>
@@ -62829,6 +63434,11 @@
       <c r="Z117" s="2"/>
       <c r="AA117" s="2"/>
       <c r="AB117" s="2"/>
+      <c r="AC117" s="2"/>
+      <c r="AD117" s="2"/>
+      <c r="AE117" s="2"/>
+      <c r="AF117" s="2"/>
+      <c r="AG117" s="2"/>
     </row>
     <row r="118" x14ac:dyDescent="0.2">
       <c r="A118" s="2"/>
@@ -62859,6 +63469,11 @@
       <c r="Z118" s="2"/>
       <c r="AA118" s="2"/>
       <c r="AB118" s="2"/>
+      <c r="AC118" s="2"/>
+      <c r="AD118" s="2"/>
+      <c r="AE118" s="2"/>
+      <c r="AF118" s="2"/>
+      <c r="AG118" s="2"/>
     </row>
     <row r="119" x14ac:dyDescent="0.2">
       <c r="A119" s="2"/>
@@ -62889,6 +63504,11 @@
       <c r="Z119" s="2"/>
       <c r="AA119" s="2"/>
       <c r="AB119" s="2"/>
+      <c r="AC119" s="2"/>
+      <c r="AD119" s="2"/>
+      <c r="AE119" s="2"/>
+      <c r="AF119" s="2"/>
+      <c r="AG119" s="2"/>
     </row>
     <row r="120" x14ac:dyDescent="0.2">
       <c r="A120" s="2"/>
@@ -62919,6 +63539,11 @@
       <c r="Z120" s="2"/>
       <c r="AA120" s="2"/>
       <c r="AB120" s="2"/>
+      <c r="AC120" s="2"/>
+      <c r="AD120" s="2"/>
+      <c r="AE120" s="2"/>
+      <c r="AF120" s="2"/>
+      <c r="AG120" s="2"/>
     </row>
     <row r="121" x14ac:dyDescent="0.2">
       <c r="A121" s="2"/>
@@ -62949,6 +63574,11 @@
       <c r="Z121" s="2"/>
       <c r="AA121" s="2"/>
       <c r="AB121" s="2"/>
+      <c r="AC121" s="2"/>
+      <c r="AD121" s="2"/>
+      <c r="AE121" s="2"/>
+      <c r="AF121" s="2"/>
+      <c r="AG121" s="2"/>
     </row>
     <row r="122" x14ac:dyDescent="0.2">
       <c r="A122" s="2"/>
@@ -62979,6 +63609,11 @@
       <c r="Z122" s="2"/>
       <c r="AA122" s="2"/>
       <c r="AB122" s="2"/>
+      <c r="AC122" s="2"/>
+      <c r="AD122" s="2"/>
+      <c r="AE122" s="2"/>
+      <c r="AF122" s="2"/>
+      <c r="AG122" s="2"/>
     </row>
     <row r="123" x14ac:dyDescent="0.2">
       <c r="A123" s="2"/>
@@ -63009,6 +63644,11 @@
       <c r="Z123" s="2"/>
       <c r="AA123" s="2"/>
       <c r="AB123" s="2"/>
+      <c r="AC123" s="2"/>
+      <c r="AD123" s="2"/>
+      <c r="AE123" s="2"/>
+      <c r="AF123" s="2"/>
+      <c r="AG123" s="2"/>
     </row>
     <row r="124" x14ac:dyDescent="0.2">
       <c r="A124" s="2"/>
@@ -63039,6 +63679,11 @@
       <c r="Z124" s="2"/>
       <c r="AA124" s="2"/>
       <c r="AB124" s="2"/>
+      <c r="AC124" s="2"/>
+      <c r="AD124" s="2"/>
+      <c r="AE124" s="2"/>
+      <c r="AF124" s="2"/>
+      <c r="AG124" s="2"/>
     </row>
     <row r="125" x14ac:dyDescent="0.2">
       <c r="A125" s="2"/>
@@ -63069,6 +63714,11 @@
       <c r="Z125" s="2"/>
       <c r="AA125" s="2"/>
       <c r="AB125" s="2"/>
+      <c r="AC125" s="2"/>
+      <c r="AD125" s="2"/>
+      <c r="AE125" s="2"/>
+      <c r="AF125" s="2"/>
+      <c r="AG125" s="2"/>
     </row>
     <row r="126" x14ac:dyDescent="0.2">
       <c r="A126" s="2"/>
@@ -63099,6 +63749,11 @@
       <c r="Z126" s="2"/>
       <c r="AA126" s="2"/>
       <c r="AB126" s="2"/>
+      <c r="AC126" s="2"/>
+      <c r="AD126" s="2"/>
+      <c r="AE126" s="2"/>
+      <c r="AF126" s="2"/>
+      <c r="AG126" s="2"/>
     </row>
     <row r="127" x14ac:dyDescent="0.2">
       <c r="A127" s="2"/>
@@ -63129,6 +63784,11 @@
       <c r="Z127" s="2"/>
       <c r="AA127" s="2"/>
       <c r="AB127" s="2"/>
+      <c r="AC127" s="2"/>
+      <c r="AD127" s="2"/>
+      <c r="AE127" s="2"/>
+      <c r="AF127" s="2"/>
+      <c r="AG127" s="2"/>
     </row>
     <row r="128" x14ac:dyDescent="0.2">
       <c r="A128" s="2"/>
@@ -63159,6 +63819,11 @@
       <c r="Z128" s="2"/>
       <c r="AA128" s="2"/>
       <c r="AB128" s="2"/>
+      <c r="AC128" s="2"/>
+      <c r="AD128" s="2"/>
+      <c r="AE128" s="2"/>
+      <c r="AF128" s="2"/>
+      <c r="AG128" s="2"/>
     </row>
     <row r="129" x14ac:dyDescent="0.2">
       <c r="A129" s="2"/>
@@ -63189,6 +63854,11 @@
       <c r="Z129" s="2"/>
       <c r="AA129" s="2"/>
       <c r="AB129" s="2"/>
+      <c r="AC129" s="2"/>
+      <c r="AD129" s="2"/>
+      <c r="AE129" s="2"/>
+      <c r="AF129" s="2"/>
+      <c r="AG129" s="2"/>
     </row>
     <row r="130" x14ac:dyDescent="0.2">
       <c r="A130" s="2"/>
@@ -63219,6 +63889,11 @@
       <c r="Z130" s="2"/>
       <c r="AA130" s="2"/>
       <c r="AB130" s="2"/>
+      <c r="AC130" s="2"/>
+      <c r="AD130" s="2"/>
+      <c r="AE130" s="2"/>
+      <c r="AF130" s="2"/>
+      <c r="AG130" s="2"/>
     </row>
     <row r="131" x14ac:dyDescent="0.2">
       <c r="A131" s="2"/>
@@ -63249,6 +63924,11 @@
       <c r="Z131" s="2"/>
       <c r="AA131" s="2"/>
       <c r="AB131" s="2"/>
+      <c r="AC131" s="2"/>
+      <c r="AD131" s="2"/>
+      <c r="AE131" s="2"/>
+      <c r="AF131" s="2"/>
+      <c r="AG131" s="2"/>
     </row>
     <row r="132" x14ac:dyDescent="0.2">
       <c r="A132" s="2"/>
@@ -63279,6 +63959,11 @@
       <c r="Z132" s="2"/>
       <c r="AA132" s="2"/>
       <c r="AB132" s="2"/>
+      <c r="AC132" s="2"/>
+      <c r="AD132" s="2"/>
+      <c r="AE132" s="2"/>
+      <c r="AF132" s="2"/>
+      <c r="AG132" s="2"/>
     </row>
     <row r="133" x14ac:dyDescent="0.2">
       <c r="A133" s="2"/>
@@ -63309,6 +63994,11 @@
       <c r="Z133" s="2"/>
       <c r="AA133" s="2"/>
       <c r="AB133" s="2"/>
+      <c r="AC133" s="2"/>
+      <c r="AD133" s="2"/>
+      <c r="AE133" s="2"/>
+      <c r="AF133" s="2"/>
+      <c r="AG133" s="2"/>
     </row>
     <row r="134" x14ac:dyDescent="0.2">
       <c r="A134" s="2"/>
@@ -63339,6 +64029,11 @@
       <c r="Z134" s="2"/>
       <c r="AA134" s="2"/>
       <c r="AB134" s="2"/>
+      <c r="AC134" s="2"/>
+      <c r="AD134" s="2"/>
+      <c r="AE134" s="2"/>
+      <c r="AF134" s="2"/>
+      <c r="AG134" s="2"/>
     </row>
     <row r="135" x14ac:dyDescent="0.2">
       <c r="A135" s="2"/>
@@ -63369,6 +64064,11 @@
       <c r="Z135" s="2"/>
       <c r="AA135" s="2"/>
       <c r="AB135" s="2"/>
+      <c r="AC135" s="2"/>
+      <c r="AD135" s="2"/>
+      <c r="AE135" s="2"/>
+      <c r="AF135" s="2"/>
+      <c r="AG135" s="2"/>
     </row>
     <row r="136" x14ac:dyDescent="0.2">
       <c r="A136" s="2"/>
@@ -63399,6 +64099,11 @@
       <c r="Z136" s="2"/>
       <c r="AA136" s="2"/>
       <c r="AB136" s="2"/>
+      <c r="AC136" s="2"/>
+      <c r="AD136" s="2"/>
+      <c r="AE136" s="2"/>
+      <c r="AF136" s="2"/>
+      <c r="AG136" s="2"/>
     </row>
     <row r="137" x14ac:dyDescent="0.2">
       <c r="A137" s="2"/>
@@ -63429,6 +64134,11 @@
       <c r="Z137" s="2"/>
       <c r="AA137" s="2"/>
       <c r="AB137" s="2"/>
+      <c r="AC137" s="2"/>
+      <c r="AD137" s="2"/>
+      <c r="AE137" s="2"/>
+      <c r="AF137" s="2"/>
+      <c r="AG137" s="2"/>
     </row>
     <row r="138" x14ac:dyDescent="0.2">
       <c r="A138" s="2"/>
@@ -63459,6 +64169,11 @@
       <c r="Z138" s="2"/>
       <c r="AA138" s="2"/>
       <c r="AB138" s="2"/>
+      <c r="AC138" s="2"/>
+      <c r="AD138" s="2"/>
+      <c r="AE138" s="2"/>
+      <c r="AF138" s="2"/>
+      <c r="AG138" s="2"/>
     </row>
     <row r="139" x14ac:dyDescent="0.2">
       <c r="A139" s="2"/>
@@ -63489,6 +64204,11 @@
       <c r="Z139" s="2"/>
       <c r="AA139" s="2"/>
       <c r="AB139" s="2"/>
+      <c r="AC139" s="2"/>
+      <c r="AD139" s="2"/>
+      <c r="AE139" s="2"/>
+      <c r="AF139" s="2"/>
+      <c r="AG139" s="2"/>
     </row>
     <row r="140" x14ac:dyDescent="0.2">
       <c r="A140" s="2"/>
@@ -63519,6 +64239,11 @@
       <c r="Z140" s="2"/>
       <c r="AA140" s="2"/>
       <c r="AB140" s="2"/>
+      <c r="AC140" s="2"/>
+      <c r="AD140" s="2"/>
+      <c r="AE140" s="2"/>
+      <c r="AF140" s="2"/>
+      <c r="AG140" s="2"/>
     </row>
     <row r="141" x14ac:dyDescent="0.2">
       <c r="A141" s="2"/>
@@ -63549,6 +64274,11 @@
       <c r="Z141" s="2"/>
       <c r="AA141" s="2"/>
       <c r="AB141" s="2"/>
+      <c r="AC141" s="2"/>
+      <c r="AD141" s="2"/>
+      <c r="AE141" s="2"/>
+      <c r="AF141" s="2"/>
+      <c r="AG141" s="2"/>
     </row>
     <row r="142" x14ac:dyDescent="0.2">
       <c r="A142" s="2"/>
@@ -63579,6 +64309,11 @@
       <c r="Z142" s="2"/>
       <c r="AA142" s="2"/>
       <c r="AB142" s="2"/>
+      <c r="AC142" s="2"/>
+      <c r="AD142" s="2"/>
+      <c r="AE142" s="2"/>
+      <c r="AF142" s="2"/>
+      <c r="AG142" s="2"/>
     </row>
     <row r="143" x14ac:dyDescent="0.2">
       <c r="A143" s="2"/>
@@ -63609,6 +64344,11 @@
       <c r="Z143" s="2"/>
       <c r="AA143" s="2"/>
       <c r="AB143" s="2"/>
+      <c r="AC143" s="2"/>
+      <c r="AD143" s="2"/>
+      <c r="AE143" s="2"/>
+      <c r="AF143" s="2"/>
+      <c r="AG143" s="2"/>
     </row>
     <row r="144" x14ac:dyDescent="0.2">
       <c r="A144" s="2"/>
@@ -63639,6 +64379,11 @@
       <c r="Z144" s="2"/>
       <c r="AA144" s="2"/>
       <c r="AB144" s="2"/>
+      <c r="AC144" s="2"/>
+      <c r="AD144" s="2"/>
+      <c r="AE144" s="2"/>
+      <c r="AF144" s="2"/>
+      <c r="AG144" s="2"/>
     </row>
     <row r="145" x14ac:dyDescent="0.2">
       <c r="A145" s="2"/>
@@ -63669,6 +64414,11 @@
       <c r="Z145" s="2"/>
       <c r="AA145" s="2"/>
       <c r="AB145" s="2"/>
+      <c r="AC145" s="2"/>
+      <c r="AD145" s="2"/>
+      <c r="AE145" s="2"/>
+      <c r="AF145" s="2"/>
+      <c r="AG145" s="2"/>
     </row>
     <row r="146" x14ac:dyDescent="0.2">
       <c r="A146" s="2"/>
@@ -63699,6 +64449,11 @@
       <c r="Z146" s="2"/>
       <c r="AA146" s="2"/>
       <c r="AB146" s="2"/>
+      <c r="AC146" s="2"/>
+      <c r="AD146" s="2"/>
+      <c r="AE146" s="2"/>
+      <c r="AF146" s="2"/>
+      <c r="AG146" s="2"/>
     </row>
     <row r="147" x14ac:dyDescent="0.2">
       <c r="A147" s="2"/>
@@ -63729,6 +64484,11 @@
       <c r="Z147" s="2"/>
       <c r="AA147" s="2"/>
       <c r="AB147" s="2"/>
+      <c r="AC147" s="2"/>
+      <c r="AD147" s="2"/>
+      <c r="AE147" s="2"/>
+      <c r="AF147" s="2"/>
+      <c r="AG147" s="2"/>
     </row>
     <row r="148" x14ac:dyDescent="0.2">
       <c r="A148" s="2"/>
@@ -63759,6 +64519,11 @@
       <c r="Z148" s="2"/>
       <c r="AA148" s="2"/>
       <c r="AB148" s="2"/>
+      <c r="AC148" s="2"/>
+      <c r="AD148" s="2"/>
+      <c r="AE148" s="2"/>
+      <c r="AF148" s="2"/>
+      <c r="AG148" s="2"/>
     </row>
     <row r="149" x14ac:dyDescent="0.2">
       <c r="A149" s="2"/>
@@ -63789,6 +64554,11 @@
       <c r="Z149" s="2"/>
       <c r="AA149" s="2"/>
       <c r="AB149" s="2"/>
+      <c r="AC149" s="2"/>
+      <c r="AD149" s="2"/>
+      <c r="AE149" s="2"/>
+      <c r="AF149" s="2"/>
+      <c r="AG149" s="2"/>
     </row>
     <row r="150" x14ac:dyDescent="0.2">
       <c r="A150" s="2"/>
@@ -63819,6 +64589,11 @@
       <c r="Z150" s="2"/>
       <c r="AA150" s="2"/>
       <c r="AB150" s="2"/>
+      <c r="AC150" s="2"/>
+      <c r="AD150" s="2"/>
+      <c r="AE150" s="2"/>
+      <c r="AF150" s="2"/>
+      <c r="AG150" s="2"/>
     </row>
     <row r="151" x14ac:dyDescent="0.2">
       <c r="A151" s="2"/>
@@ -63849,6 +64624,11 @@
       <c r="Z151" s="2"/>
       <c r="AA151" s="2"/>
       <c r="AB151" s="2"/>
+      <c r="AC151" s="2"/>
+      <c r="AD151" s="2"/>
+      <c r="AE151" s="2"/>
+      <c r="AF151" s="2"/>
+      <c r="AG151" s="2"/>
     </row>
     <row r="152" x14ac:dyDescent="0.2">
       <c r="A152" s="2"/>
@@ -63879,6 +64659,11 @@
       <c r="Z152" s="2"/>
       <c r="AA152" s="2"/>
       <c r="AB152" s="2"/>
+      <c r="AC152" s="2"/>
+      <c r="AD152" s="2"/>
+      <c r="AE152" s="2"/>
+      <c r="AF152" s="2"/>
+      <c r="AG152" s="2"/>
     </row>
     <row r="153" x14ac:dyDescent="0.2">
       <c r="A153" s="2"/>
@@ -63909,6 +64694,11 @@
       <c r="Z153" s="2"/>
       <c r="AA153" s="2"/>
       <c r="AB153" s="2"/>
+      <c r="AC153" s="2"/>
+      <c r="AD153" s="2"/>
+      <c r="AE153" s="2"/>
+      <c r="AF153" s="2"/>
+      <c r="AG153" s="2"/>
     </row>
     <row r="154" x14ac:dyDescent="0.2">
       <c r="A154" s="2"/>
@@ -63939,6 +64729,11 @@
       <c r="Z154" s="2"/>
       <c r="AA154" s="2"/>
       <c r="AB154" s="2"/>
+      <c r="AC154" s="2"/>
+      <c r="AD154" s="2"/>
+      <c r="AE154" s="2"/>
+      <c r="AF154" s="2"/>
+      <c r="AG154" s="2"/>
     </row>
     <row r="155" x14ac:dyDescent="0.2">
       <c r="A155" s="2"/>
@@ -63969,6 +64764,11 @@
       <c r="Z155" s="2"/>
       <c r="AA155" s="2"/>
       <c r="AB155" s="2"/>
+      <c r="AC155" s="2"/>
+      <c r="AD155" s="2"/>
+      <c r="AE155" s="2"/>
+      <c r="AF155" s="2"/>
+      <c r="AG155" s="2"/>
     </row>
     <row r="156" x14ac:dyDescent="0.2">
       <c r="A156" s="2"/>
@@ -63999,6 +64799,11 @@
       <c r="Z156" s="2"/>
       <c r="AA156" s="2"/>
       <c r="AB156" s="2"/>
+      <c r="AC156" s="2"/>
+      <c r="AD156" s="2"/>
+      <c r="AE156" s="2"/>
+      <c r="AF156" s="2"/>
+      <c r="AG156" s="2"/>
     </row>
     <row r="157" x14ac:dyDescent="0.2">
       <c r="A157" s="2"/>
@@ -64029,6 +64834,11 @@
       <c r="Z157" s="2"/>
       <c r="AA157" s="2"/>
       <c r="AB157" s="2"/>
+      <c r="AC157" s="2"/>
+      <c r="AD157" s="2"/>
+      <c r="AE157" s="2"/>
+      <c r="AF157" s="2"/>
+      <c r="AG157" s="2"/>
     </row>
     <row r="158" x14ac:dyDescent="0.2">
       <c r="A158" s="2"/>
@@ -64059,6 +64869,11 @@
       <c r="Z158" s="2"/>
       <c r="AA158" s="2"/>
       <c r="AB158" s="2"/>
+      <c r="AC158" s="2"/>
+      <c r="AD158" s="2"/>
+      <c r="AE158" s="2"/>
+      <c r="AF158" s="2"/>
+      <c r="AG158" s="2"/>
     </row>
     <row r="159" x14ac:dyDescent="0.2">
       <c r="A159" s="2"/>
@@ -64089,6 +64904,11 @@
       <c r="Z159" s="2"/>
       <c r="AA159" s="2"/>
       <c r="AB159" s="2"/>
+      <c r="AC159" s="2"/>
+      <c r="AD159" s="2"/>
+      <c r="AE159" s="2"/>
+      <c r="AF159" s="2"/>
+      <c r="AG159" s="2"/>
     </row>
     <row r="160" x14ac:dyDescent="0.2">
       <c r="A160" s="2"/>
@@ -64119,6 +64939,11 @@
       <c r="Z160" s="2"/>
       <c r="AA160" s="2"/>
       <c r="AB160" s="2"/>
+      <c r="AC160" s="2"/>
+      <c r="AD160" s="2"/>
+      <c r="AE160" s="2"/>
+      <c r="AF160" s="2"/>
+      <c r="AG160" s="2"/>
     </row>
     <row r="161" x14ac:dyDescent="0.2">
       <c r="A161" s="2"/>
@@ -64149,6 +64974,11 @@
       <c r="Z161" s="2"/>
       <c r="AA161" s="2"/>
       <c r="AB161" s="2"/>
+      <c r="AC161" s="2"/>
+      <c r="AD161" s="2"/>
+      <c r="AE161" s="2"/>
+      <c r="AF161" s="2"/>
+      <c r="AG161" s="2"/>
     </row>
     <row r="162" x14ac:dyDescent="0.2">
       <c r="A162" s="2"/>
@@ -64179,6 +65009,11 @@
       <c r="Z162" s="2"/>
       <c r="AA162" s="2"/>
       <c r="AB162" s="2"/>
+      <c r="AC162" s="2"/>
+      <c r="AD162" s="2"/>
+      <c r="AE162" s="2"/>
+      <c r="AF162" s="2"/>
+      <c r="AG162" s="2"/>
     </row>
     <row r="163" x14ac:dyDescent="0.2">
       <c r="A163" s="2"/>
@@ -64209,6 +65044,11 @@
       <c r="Z163" s="2"/>
       <c r="AA163" s="2"/>
       <c r="AB163" s="2"/>
+      <c r="AC163" s="2"/>
+      <c r="AD163" s="2"/>
+      <c r="AE163" s="2"/>
+      <c r="AF163" s="2"/>
+      <c r="AG163" s="2"/>
     </row>
     <row r="164" x14ac:dyDescent="0.2">
       <c r="A164" s="2"/>
@@ -64239,6 +65079,11 @@
       <c r="Z164" s="2"/>
       <c r="AA164" s="2"/>
       <c r="AB164" s="2"/>
+      <c r="AC164" s="2"/>
+      <c r="AD164" s="2"/>
+      <c r="AE164" s="2"/>
+      <c r="AF164" s="2"/>
+      <c r="AG164" s="2"/>
     </row>
     <row r="165" x14ac:dyDescent="0.2">
       <c r="A165" s="2"/>
@@ -64269,6 +65114,11 @@
       <c r="Z165" s="2"/>
       <c r="AA165" s="2"/>
       <c r="AB165" s="2"/>
+      <c r="AC165" s="2"/>
+      <c r="AD165" s="2"/>
+      <c r="AE165" s="2"/>
+      <c r="AF165" s="2"/>
+      <c r="AG165" s="2"/>
     </row>
     <row r="166" x14ac:dyDescent="0.2">
       <c r="A166" s="2"/>
@@ -64299,6 +65149,11 @@
       <c r="Z166" s="2"/>
       <c r="AA166" s="2"/>
       <c r="AB166" s="2"/>
+      <c r="AC166" s="2"/>
+      <c r="AD166" s="2"/>
+      <c r="AE166" s="2"/>
+      <c r="AF166" s="2"/>
+      <c r="AG166" s="2"/>
     </row>
     <row r="167" x14ac:dyDescent="0.2">
       <c r="A167" s="2"/>
@@ -64329,6 +65184,11 @@
       <c r="Z167" s="2"/>
       <c r="AA167" s="2"/>
       <c r="AB167" s="2"/>
+      <c r="AC167" s="2"/>
+      <c r="AD167" s="2"/>
+      <c r="AE167" s="2"/>
+      <c r="AF167" s="2"/>
+      <c r="AG167" s="2"/>
     </row>
     <row r="168" x14ac:dyDescent="0.2">
       <c r="A168" s="2"/>
@@ -64359,6 +65219,11 @@
       <c r="Z168" s="2"/>
       <c r="AA168" s="2"/>
       <c r="AB168" s="2"/>
+      <c r="AC168" s="2"/>
+      <c r="AD168" s="2"/>
+      <c r="AE168" s="2"/>
+      <c r="AF168" s="2"/>
+      <c r="AG168" s="2"/>
     </row>
     <row r="169" x14ac:dyDescent="0.2">
       <c r="A169" s="2"/>
@@ -64389,6 +65254,11 @@
       <c r="Z169" s="2"/>
       <c r="AA169" s="2"/>
       <c r="AB169" s="2"/>
+      <c r="AC169" s="2"/>
+      <c r="AD169" s="2"/>
+      <c r="AE169" s="2"/>
+      <c r="AF169" s="2"/>
+      <c r="AG169" s="2"/>
     </row>
     <row r="170" x14ac:dyDescent="0.2">
       <c r="A170" s="2"/>
@@ -64419,6 +65289,11 @@
       <c r="Z170" s="2"/>
       <c r="AA170" s="2"/>
       <c r="AB170" s="2"/>
+      <c r="AC170" s="2"/>
+      <c r="AD170" s="2"/>
+      <c r="AE170" s="2"/>
+      <c r="AF170" s="2"/>
+      <c r="AG170" s="2"/>
     </row>
     <row r="171" x14ac:dyDescent="0.2">
       <c r="A171" s="2"/>
@@ -64449,6 +65324,11 @@
       <c r="Z171" s="2"/>
       <c r="AA171" s="2"/>
       <c r="AB171" s="2"/>
+      <c r="AC171" s="2"/>
+      <c r="AD171" s="2"/>
+      <c r="AE171" s="2"/>
+      <c r="AF171" s="2"/>
+      <c r="AG171" s="2"/>
     </row>
     <row r="172" x14ac:dyDescent="0.2">
       <c r="A172" s="2"/>
@@ -64479,6 +65359,11 @@
       <c r="Z172" s="2"/>
       <c r="AA172" s="2"/>
       <c r="AB172" s="2"/>
+      <c r="AC172" s="2"/>
+      <c r="AD172" s="2"/>
+      <c r="AE172" s="2"/>
+      <c r="AF172" s="2"/>
+      <c r="AG172" s="2"/>
     </row>
     <row r="173" x14ac:dyDescent="0.2">
       <c r="A173" s="2"/>
@@ -64509,6 +65394,11 @@
       <c r="Z173" s="2"/>
       <c r="AA173" s="2"/>
       <c r="AB173" s="2"/>
+      <c r="AC173" s="2"/>
+      <c r="AD173" s="2"/>
+      <c r="AE173" s="2"/>
+      <c r="AF173" s="2"/>
+      <c r="AG173" s="2"/>
     </row>
     <row r="174" x14ac:dyDescent="0.2">
       <c r="A174" s="2"/>
@@ -64539,6 +65429,11 @@
       <c r="Z174" s="2"/>
       <c r="AA174" s="2"/>
       <c r="AB174" s="2"/>
+      <c r="AC174" s="2"/>
+      <c r="AD174" s="2"/>
+      <c r="AE174" s="2"/>
+      <c r="AF174" s="2"/>
+      <c r="AG174" s="2"/>
     </row>
     <row r="175" x14ac:dyDescent="0.2">
       <c r="A175" s="2"/>
@@ -64569,6 +65464,11 @@
       <c r="Z175" s="2"/>
       <c r="AA175" s="2"/>
       <c r="AB175" s="2"/>
+      <c r="AC175" s="2"/>
+      <c r="AD175" s="2"/>
+      <c r="AE175" s="2"/>
+      <c r="AF175" s="2"/>
+      <c r="AG175" s="2"/>
     </row>
     <row r="176" x14ac:dyDescent="0.2">
       <c r="A176" s="2"/>
@@ -64599,6 +65499,11 @@
       <c r="Z176" s="2"/>
       <c r="AA176" s="2"/>
       <c r="AB176" s="2"/>
+      <c r="AC176" s="2"/>
+      <c r="AD176" s="2"/>
+      <c r="AE176" s="2"/>
+      <c r="AF176" s="2"/>
+      <c r="AG176" s="2"/>
     </row>
     <row r="177" x14ac:dyDescent="0.2">
       <c r="A177" s="2"/>
@@ -64629,6 +65534,11 @@
       <c r="Z177" s="2"/>
       <c r="AA177" s="2"/>
       <c r="AB177" s="2"/>
+      <c r="AC177" s="2"/>
+      <c r="AD177" s="2"/>
+      <c r="AE177" s="2"/>
+      <c r="AF177" s="2"/>
+      <c r="AG177" s="2"/>
     </row>
     <row r="178" x14ac:dyDescent="0.2">
       <c r="A178" s="2"/>
@@ -64659,6 +65569,11 @@
       <c r="Z178" s="2"/>
       <c r="AA178" s="2"/>
       <c r="AB178" s="2"/>
+      <c r="AC178" s="2"/>
+      <c r="AD178" s="2"/>
+      <c r="AE178" s="2"/>
+      <c r="AF178" s="2"/>
+      <c r="AG178" s="2"/>
     </row>
     <row r="179" x14ac:dyDescent="0.2">
       <c r="A179" s="2"/>
@@ -64689,6 +65604,11 @@
       <c r="Z179" s="2"/>
       <c r="AA179" s="2"/>
       <c r="AB179" s="2"/>
+      <c r="AC179" s="2"/>
+      <c r="AD179" s="2"/>
+      <c r="AE179" s="2"/>
+      <c r="AF179" s="2"/>
+      <c r="AG179" s="2"/>
     </row>
     <row r="180" x14ac:dyDescent="0.2">
       <c r="A180" s="2"/>
@@ -64719,6 +65639,11 @@
       <c r="Z180" s="2"/>
       <c r="AA180" s="2"/>
       <c r="AB180" s="2"/>
+      <c r="AC180" s="2"/>
+      <c r="AD180" s="2"/>
+      <c r="AE180" s="2"/>
+      <c r="AF180" s="2"/>
+      <c r="AG180" s="2"/>
     </row>
     <row r="181" x14ac:dyDescent="0.2">
       <c r="A181" s="2"/>
@@ -64749,6 +65674,11 @@
       <c r="Z181" s="2"/>
       <c r="AA181" s="2"/>
       <c r="AB181" s="2"/>
+      <c r="AC181" s="2"/>
+      <c r="AD181" s="2"/>
+      <c r="AE181" s="2"/>
+      <c r="AF181" s="2"/>
+      <c r="AG181" s="2"/>
     </row>
     <row r="182" x14ac:dyDescent="0.2">
       <c r="A182" s="2"/>
@@ -64779,6 +65709,11 @@
       <c r="Z182" s="2"/>
       <c r="AA182" s="2"/>
       <c r="AB182" s="2"/>
+      <c r="AC182" s="2"/>
+      <c r="AD182" s="2"/>
+      <c r="AE182" s="2"/>
+      <c r="AF182" s="2"/>
+      <c r="AG182" s="2"/>
     </row>
     <row r="183" x14ac:dyDescent="0.2">
       <c r="A183" s="2"/>
@@ -64809,6 +65744,11 @@
       <c r="Z183" s="2"/>
       <c r="AA183" s="2"/>
       <c r="AB183" s="2"/>
+      <c r="AC183" s="2"/>
+      <c r="AD183" s="2"/>
+      <c r="AE183" s="2"/>
+      <c r="AF183" s="2"/>
+      <c r="AG183" s="2"/>
     </row>
     <row r="184" x14ac:dyDescent="0.2">
       <c r="A184" s="2"/>
@@ -64839,6 +65779,11 @@
       <c r="Z184" s="2"/>
       <c r="AA184" s="2"/>
       <c r="AB184" s="2"/>
+      <c r="AC184" s="2"/>
+      <c r="AD184" s="2"/>
+      <c r="AE184" s="2"/>
+      <c r="AF184" s="2"/>
+      <c r="AG184" s="2"/>
     </row>
     <row r="185" x14ac:dyDescent="0.2">
       <c r="A185" s="2"/>
@@ -64869,6 +65814,11 @@
       <c r="Z185" s="2"/>
       <c r="AA185" s="2"/>
       <c r="AB185" s="2"/>
+      <c r="AC185" s="2"/>
+      <c r="AD185" s="2"/>
+      <c r="AE185" s="2"/>
+      <c r="AF185" s="2"/>
+      <c r="AG185" s="2"/>
     </row>
     <row r="186" x14ac:dyDescent="0.2">
       <c r="A186" s="2"/>
@@ -64899,6 +65849,11 @@
       <c r="Z186" s="2"/>
       <c r="AA186" s="2"/>
       <c r="AB186" s="2"/>
+      <c r="AC186" s="2"/>
+      <c r="AD186" s="2"/>
+      <c r="AE186" s="2"/>
+      <c r="AF186" s="2"/>
+      <c r="AG186" s="2"/>
     </row>
     <row r="187" x14ac:dyDescent="0.2">
       <c r="A187" s="2"/>
@@ -64929,6 +65884,11 @@
       <c r="Z187" s="2"/>
       <c r="AA187" s="2"/>
       <c r="AB187" s="2"/>
+      <c r="AC187" s="2"/>
+      <c r="AD187" s="2"/>
+      <c r="AE187" s="2"/>
+      <c r="AF187" s="2"/>
+      <c r="AG187" s="2"/>
     </row>
     <row r="188" x14ac:dyDescent="0.2">
       <c r="A188" s="2"/>
@@ -64959,6 +65919,11 @@
       <c r="Z188" s="2"/>
       <c r="AA188" s="2"/>
       <c r="AB188" s="2"/>
+      <c r="AC188" s="2"/>
+      <c r="AD188" s="2"/>
+      <c r="AE188" s="2"/>
+      <c r="AF188" s="2"/>
+      <c r="AG188" s="2"/>
     </row>
     <row r="189" x14ac:dyDescent="0.2">
       <c r="A189" s="2"/>
@@ -64989,6 +65954,11 @@
       <c r="Z189" s="2"/>
       <c r="AA189" s="2"/>
       <c r="AB189" s="2"/>
+      <c r="AC189" s="2"/>
+      <c r="AD189" s="2"/>
+      <c r="AE189" s="2"/>
+      <c r="AF189" s="2"/>
+      <c r="AG189" s="2"/>
     </row>
     <row r="190" x14ac:dyDescent="0.2">
       <c r="A190" s="2"/>
@@ -65019,6 +65989,11 @@
       <c r="Z190" s="2"/>
       <c r="AA190" s="2"/>
       <c r="AB190" s="2"/>
+      <c r="AC190" s="2"/>
+      <c r="AD190" s="2"/>
+      <c r="AE190" s="2"/>
+      <c r="AF190" s="2"/>
+      <c r="AG190" s="2"/>
     </row>
     <row r="191" x14ac:dyDescent="0.2">
       <c r="A191" s="2"/>
@@ -65049,6 +66024,11 @@
       <c r="Z191" s="2"/>
       <c r="AA191" s="2"/>
       <c r="AB191" s="2"/>
+      <c r="AC191" s="2"/>
+      <c r="AD191" s="2"/>
+      <c r="AE191" s="2"/>
+      <c r="AF191" s="2"/>
+      <c r="AG191" s="2"/>
     </row>
     <row r="192" x14ac:dyDescent="0.2">
       <c r="A192" s="2"/>
@@ -65079,6 +66059,11 @@
       <c r="Z192" s="2"/>
       <c r="AA192" s="2"/>
       <c r="AB192" s="2"/>
+      <c r="AC192" s="2"/>
+      <c r="AD192" s="2"/>
+      <c r="AE192" s="2"/>
+      <c r="AF192" s="2"/>
+      <c r="AG192" s="2"/>
     </row>
     <row r="193" x14ac:dyDescent="0.2">
       <c r="A193" s="2"/>
@@ -65109,6 +66094,11 @@
       <c r="Z193" s="2"/>
       <c r="AA193" s="2"/>
       <c r="AB193" s="2"/>
+      <c r="AC193" s="2"/>
+      <c r="AD193" s="2"/>
+      <c r="AE193" s="2"/>
+      <c r="AF193" s="2"/>
+      <c r="AG193" s="2"/>
     </row>
     <row r="194" x14ac:dyDescent="0.2">
       <c r="A194" s="2"/>
@@ -65139,6 +66129,11 @@
       <c r="Z194" s="2"/>
       <c r="AA194" s="2"/>
       <c r="AB194" s="2"/>
+      <c r="AC194" s="2"/>
+      <c r="AD194" s="2"/>
+      <c r="AE194" s="2"/>
+      <c r="AF194" s="2"/>
+      <c r="AG194" s="2"/>
     </row>
     <row r="195" x14ac:dyDescent="0.2">
       <c r="A195" s="2"/>
@@ -65169,6 +66164,11 @@
       <c r="Z195" s="2"/>
       <c r="AA195" s="2"/>
       <c r="AB195" s="2"/>
+      <c r="AC195" s="2"/>
+      <c r="AD195" s="2"/>
+      <c r="AE195" s="2"/>
+      <c r="AF195" s="2"/>
+      <c r="AG195" s="2"/>
     </row>
     <row r="196" x14ac:dyDescent="0.2">
       <c r="A196" s="2"/>
@@ -65199,6 +66199,11 @@
       <c r="Z196" s="2"/>
       <c r="AA196" s="2"/>
       <c r="AB196" s="2"/>
+      <c r="AC196" s="2"/>
+      <c r="AD196" s="2"/>
+      <c r="AE196" s="2"/>
+      <c r="AF196" s="2"/>
+      <c r="AG196" s="2"/>
     </row>
     <row r="197" x14ac:dyDescent="0.2">
       <c r="A197" s="2"/>
@@ -65229,6 +66234,11 @@
       <c r="Z197" s="2"/>
       <c r="AA197" s="2"/>
       <c r="AB197" s="2"/>
+      <c r="AC197" s="2"/>
+      <c r="AD197" s="2"/>
+      <c r="AE197" s="2"/>
+      <c r="AF197" s="2"/>
+      <c r="AG197" s="2"/>
     </row>
     <row r="198" x14ac:dyDescent="0.2">
       <c r="A198" s="2"/>
@@ -65259,6 +66269,11 @@
       <c r="Z198" s="2"/>
       <c r="AA198" s="2"/>
       <c r="AB198" s="2"/>
+      <c r="AC198" s="2"/>
+      <c r="AD198" s="2"/>
+      <c r="AE198" s="2"/>
+      <c r="AF198" s="2"/>
+      <c r="AG198" s="2"/>
     </row>
     <row r="199" x14ac:dyDescent="0.2">
       <c r="A199" s="2"/>
@@ -65289,6 +66304,11 @@
       <c r="Z199" s="2"/>
       <c r="AA199" s="2"/>
       <c r="AB199" s="2"/>
+      <c r="AC199" s="2"/>
+      <c r="AD199" s="2"/>
+      <c r="AE199" s="2"/>
+      <c r="AF199" s="2"/>
+      <c r="AG199" s="2"/>
     </row>
     <row r="200" x14ac:dyDescent="0.2">
       <c r="A200" s="2"/>
@@ -65319,6 +66339,11 @@
       <c r="Z200" s="2"/>
       <c r="AA200" s="2"/>
       <c r="AB200" s="2"/>
+      <c r="AC200" s="2"/>
+      <c r="AD200" s="2"/>
+      <c r="AE200" s="2"/>
+      <c r="AF200" s="2"/>
+      <c r="AG200" s="2"/>
     </row>
     <row r="201" x14ac:dyDescent="0.2">
       <c r="A201" s="2"/>
@@ -65349,6 +66374,11 @@
       <c r="Z201" s="2"/>
       <c r="AA201" s="2"/>
       <c r="AB201" s="2"/>
+      <c r="AC201" s="2"/>
+      <c r="AD201" s="2"/>
+      <c r="AE201" s="2"/>
+      <c r="AF201" s="2"/>
+      <c r="AG201" s="2"/>
     </row>
     <row r="202" x14ac:dyDescent="0.2">
       <c r="A202" s="2"/>
@@ -65379,47 +66409,62 @@
       <c r="Z202" s="2"/>
       <c r="AA202" s="2"/>
       <c r="AB202" s="2"/>
+      <c r="AC202" s="2"/>
+      <c r="AD202" s="2"/>
+      <c r="AE202" s="2"/>
+      <c r="AF202" s="2"/>
+      <c r="AG202" s="2"/>
     </row>
     <row r="203" x14ac:dyDescent="0.2">
       <c r="A203" s="2"/>
       <c r="B203" s="59"/>
+      <c r="R203" s="2"/>
+      <c r="S203" s="2"/>
+      <c r="T203" s="2"/>
+      <c r="U203" s="2"/>
+      <c r="W203" s="2"/>
     </row>
   </sheetData>
   <sheetProtection algorithmName="SHA-512" hashValue="FpwA99+lZ3tcetgbufn/FDC8HQLhHeenUtUDopBd7olIgbOkNoNGn9spTr6VyjbhJ25LGDZVYLCeDv+4Ep88iQ==" saltValue="ZbPAwiTrvBPOJT2KMdL6dA==" spinCount="100000" sheet="1" selectLockedCells="1"/>
-  <mergeCells count="20">
+  <mergeCells count="25">
     <mergeCell ref="F2:F3"/>
     <mergeCell ref="G2:H2"/>
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="C1:E1"/>
     <mergeCell ref="A1:A3"/>
     <mergeCell ref="B1:B3"/>
-    <mergeCell ref="X1:X3"/>
-    <mergeCell ref="Y1:AB2"/>
-    <mergeCell ref="U1:V2"/>
-    <mergeCell ref="W1:W3"/>
+    <mergeCell ref="AC1:AC3"/>
+    <mergeCell ref="AD1:AG2"/>
+    <mergeCell ref="Z1:AA2"/>
+    <mergeCell ref="AB1:AB3"/>
     <mergeCell ref="K1:M2"/>
     <mergeCell ref="P1:P3"/>
     <mergeCell ref="Q1:Q3"/>
-    <mergeCell ref="R1:R3"/>
-    <mergeCell ref="S1:T2"/>
+    <mergeCell ref="V1:V3"/>
+    <mergeCell ref="X1:Y2"/>
     <mergeCell ref="I1:I3"/>
     <mergeCell ref="J1:J3"/>
     <mergeCell ref="N1:O2"/>
     <mergeCell ref="C2:C3"/>
     <mergeCell ref="D2:E2"/>
+    <mergeCell ref="R1:R3"/>
+    <mergeCell ref="S1:S3"/>
+    <mergeCell ref="T1:T3"/>
+    <mergeCell ref="U1:U3"/>
+    <mergeCell ref="W1:W3"/>
   </mergeCells>
   <dataValidations count="1">
-    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3 Y3:AB3" xr:uid="{BB3B8D3D-2F24-4FC4-9101-48D8CFEF3D7F}">
+    <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="K3 AD3:AG3" xr:uid="{BB3B8D3D-2F24-4FC4-9101-48D8CFEF3D7F}">
       <formula1>"&lt;0&gt;0"</formula1>
     </dataValidation>
   </dataValidations>
   <hyperlinks>
-    <hyperlink ref="Y3" r:id="rIdSpecies420_1" xr:uid="{2BC6450F-A7B4-4044-BEA6-59E54066E449}" location="allSpecies"/>
-    <hyperlink ref="Z3" r:id="rIdSpecies420_2" xr:uid="{9EEA8352-0631-4B4E-BB1B-FF880D8B8ED2}" location="allSpecies"/>
-    <hyperlink ref="AA3" r:id="rIdSpecies420_3" xr:uid="{B78A1E77-3003-40C6-9B0C-101A94179479}" location="allSpecies"/>
-    <hyperlink ref="AB3" r:id="rIdSpecies420_4" xr:uid="{22DD36F0-D891-4763-8CC9-508C73D63CC9}" location="allSpecies"/>
+    <hyperlink ref="AD3" r:id="rIdSpecies420_1" xr:uid="{2BC6450F-A7B4-4044-BEA6-59E54066E449}" location="allSpecies"/>
+    <hyperlink ref="AE3" r:id="rIdSpecies420_2" xr:uid="{9EEA8352-0631-4B4E-BB1B-FF880D8B8ED2}" location="allSpecies"/>
+    <hyperlink ref="AF3" r:id="rIdSpecies420_3" xr:uid="{B78A1E77-3003-40C6-9B0C-101A94179479}" location="allSpecies"/>
+    <hyperlink ref="AG3" r:id="rIdSpecies420_4" xr:uid="{22DD36F0-D891-4763-8CC9-508C73D63CC9}" location="allSpecies"/>
     <hyperlink ref="K3" r:id="rId5" location="lineMaterialTypes" xr:uid="{53874CDA-60F7-44F3-A738-546AA82ACA2B}"/>
-    <hyperlink ref="U3" r:id="rId6" location="lineMaterialTypes" xr:uid="{7EF57AEF-2AD1-4676-A048-1EB51C0592B2}"/>
+    <hyperlink ref="Z3" r:id="rId6" location="lineMaterialTypes" xr:uid="{7EF57AEF-2AD1-4676-A048-1EB51C0592B2}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>